<commit_message>
update Testcase-OrangeHRM.xlsx with new data
</commit_message>
<xml_diff>
--- a/Testcase-OrangeHRM.xlsx
+++ b/Testcase-OrangeHRM.xlsx
@@ -9,8 +9,7 @@
     <sheet state="visible" name="Danh sách nhân viên" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Đăng nhập'!$A$2:$J$27</definedName>
-    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Quản lý người dùng'!$A$2:$J$28</definedName>
+    <definedName hidden="1" localSheetId="2" name="_xlnm._FilterDatabase">'Quản lý người dùng'!$A$2:$J$29</definedName>
     <definedName hidden="1" localSheetId="3" name="_xlnm._FilterDatabase">'Danh sách nhân viên'!$A$2:$J$29</definedName>
   </definedNames>
   <calcPr/>
@@ -18,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="461">
   <si>
     <t>MA TRẬN KIỂM THỬ – KIỂM THỬ TỰ ĐỘNG ORANGEHRM (Playwright)</t>
   </si>
@@ -561,6 +560,9 @@
     <t>Bảng danh sách hiển thị với các cột: Tên tài khoản, Vai trò, Tên nhân viên, Trạng thái</t>
   </si>
   <si>
+    <t>Passed</t>
+  </si>
+  <si>
     <t>Kiểm tra 4 tiêu đề cột tồn tại</t>
   </si>
   <si>
@@ -705,10 +707,30 @@
     <t>Kiểm tra ô tìm kiếm đã trống sau khi xóa bộ lọc</t>
   </si>
   <si>
+    <t>TC-U08</t>
+  </si>
+  <si>
+    <t>Tìm kiếm tên tài khoản chỉ gồm khoảng trắng</t>
+  </si>
+  <si>
+    <t>Hệ thống không trả về kết quả khi từ khóa tìm kiếm chỉ là khoảng trắng</t>
+  </si>
+  <si>
+    <t>1. Vào Quản lý người dùng
+2. Nhập 3 dấu cách vào ô Tên tài khoản
+3. Nhấn Tìm kiếm</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Trung bình</t>
+  </si>
+  <si>
+    <t>Observed on 2026-06-06: nhập khoảng trắng và Search vẫn hiển thị (10) Records Found</t>
+  </si>
+  <si>
     <t>Thêm người dùng mới</t>
-  </si>
-  <si>
-    <t>TC-U08</t>
   </si>
   <si>
     <t>Thêm người dùng mới với thông tin đầy đủ và hợp lệ</t>
@@ -1687,7 +1709,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -1757,6 +1779,11 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="13">
@@ -1962,7 +1989,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="47">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2009,6 +2036,9 @@
     <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="4" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="8" fillId="10" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2017,14 +2047,14 @@
     <xf borderId="11" fillId="11" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="11" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
     <xf borderId="11" fillId="8" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="11" fillId="8" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="11" fillId="11" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -2059,8 +2089,23 @@
     <xf borderId="4" fillId="11" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="4" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="4" fillId="8" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="6" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="8" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="7" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="12" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -3518,8 +3563,7 @@
     <col customWidth="1" min="4" max="4" width="28.0"/>
     <col customWidth="1" min="5" max="5" width="46.0"/>
     <col customWidth="1" min="6" max="6" width="44.0"/>
-    <col customWidth="1" min="7" max="7" width="20.0"/>
-    <col customWidth="1" min="8" max="8" width="14.0"/>
+    <col customWidth="1" min="7" max="8" width="20.0"/>
     <col customWidth="1" min="9" max="9" width="13.0"/>
     <col customWidth="1" min="10" max="10" width="34.0"/>
     <col customWidth="1" min="11" max="26" width="8.71"/>
@@ -3561,7 +3605,7 @@
       <c r="G2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="18" t="s">
         <v>41</v>
       </c>
       <c r="I2" s="5" t="s">
@@ -3572,46 +3616,46 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="21"/>
     </row>
     <row r="4" ht="69.75" customHeight="1">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="22" t="s">
+      <c r="G4" s="22"/>
+      <c r="H4" s="9" t="s">
         <v>51</v>
       </c>
       <c r="I4" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="21" t="s">
+      <c r="J4" s="22" t="s">
         <v>53</v>
       </c>
     </row>
@@ -3635,7 +3679,7 @@
         <v>59</v>
       </c>
       <c r="G5" s="24"/>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I5" s="23" t="s">
@@ -3646,32 +3690,32 @@
       </c>
     </row>
     <row r="6" ht="69.75" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="G6" s="21"/>
-      <c r="H6" s="22" t="s">
+      <c r="G6" s="22"/>
+      <c r="H6" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I6" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="J6" s="22" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3695,7 +3739,7 @@
         <v>73</v>
       </c>
       <c r="G7" s="24"/>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I7" s="23" t="s">
@@ -3706,32 +3750,32 @@
       </c>
     </row>
     <row r="8" ht="69.75" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="F8" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="22" t="s">
+      <c r="G8" s="22"/>
+      <c r="H8" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I8" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="22" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3755,7 +3799,7 @@
         <v>87</v>
       </c>
       <c r="G9" s="24"/>
-      <c r="H9" s="22" t="s">
+      <c r="H9" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I9" s="23" t="s">
@@ -3766,18 +3810,18 @@
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="11" ht="69.75" customHeight="1">
       <c r="A11" s="24" t="s">
@@ -3799,7 +3843,7 @@
         <v>94</v>
       </c>
       <c r="G11" s="24"/>
-      <c r="H11" s="22" t="s">
+      <c r="H11" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I11" s="23" t="s">
@@ -3810,32 +3854,32 @@
       </c>
     </row>
     <row r="12" ht="69.75" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="22" t="s">
         <v>101</v>
       </c>
-      <c r="G12" s="21"/>
-      <c r="H12" s="29" t="s">
+      <c r="G12" s="22"/>
+      <c r="H12" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="I12" s="30" t="s">
+      <c r="I12" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="J12" s="25" t="s">
+      <c r="J12" s="26" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3852,14 +3896,14 @@
       <c r="D13" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="E13" s="31" t="s">
+      <c r="E13" s="32" t="s">
         <v>109</v>
       </c>
       <c r="F13" s="24" t="s">
         <v>110</v>
       </c>
       <c r="G13" s="24"/>
-      <c r="H13" s="22" t="s">
+      <c r="H13" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I13" s="23" t="s">
@@ -3870,76 +3914,76 @@
       </c>
     </row>
     <row r="14" ht="69.75" customHeight="1">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="F14" s="25" t="s">
+      <c r="F14" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="G14" s="21"/>
-      <c r="H14" s="29" t="s">
+      <c r="G14" s="22"/>
+      <c r="H14" s="30" t="s">
         <v>102</v>
       </c>
-      <c r="I14" s="30" t="s">
+      <c r="I14" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="J14" s="25" t="s">
+      <c r="J14" s="26" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="26" t="s">
+      <c r="A15" s="27" t="s">
         <v>119</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="29"/>
     </row>
     <row r="16" ht="69.75" customHeight="1">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="22" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="22" t="s">
         <v>124</v>
       </c>
-      <c r="F16" s="21" t="s">
+      <c r="F16" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="G16" s="21"/>
-      <c r="H16" s="22" t="s">
+      <c r="G16" s="22"/>
+      <c r="H16" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I16" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J16" s="21" t="s">
+      <c r="J16" s="22" t="s">
         <v>126</v>
       </c>
     </row>
@@ -3963,7 +4007,7 @@
         <v>131</v>
       </c>
       <c r="G17" s="24"/>
-      <c r="H17" s="22" t="s">
+      <c r="H17" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I17" s="23" t="s">
@@ -3974,32 +4018,32 @@
       </c>
     </row>
     <row r="18" ht="69.75" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="D18" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="E18" s="21" t="s">
+      <c r="E18" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="G18" s="21"/>
-      <c r="H18" s="22" t="s">
+      <c r="G18" s="22"/>
+      <c r="H18" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I18" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J18" s="21" t="s">
+      <c r="J18" s="22" t="s">
         <v>139</v>
       </c>
     </row>
@@ -4013,7 +4057,7 @@
       <c r="C19" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="D19" s="31" t="s">
+      <c r="D19" s="32" t="s">
         <v>143</v>
       </c>
       <c r="E19" s="24" t="s">
@@ -4023,7 +4067,7 @@
         <v>145</v>
       </c>
       <c r="G19" s="24"/>
-      <c r="H19" s="22" t="s">
+      <c r="H19" s="25" t="s">
         <v>51</v>
       </c>
       <c r="I19" s="23" t="s">
@@ -4034,118 +4078,118 @@
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="33" t="s">
+      <c r="A20" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="29"/>
     </row>
     <row r="21" ht="69.75" customHeight="1">
       <c r="A21" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="32" t="s">
         <v>149</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="D21" s="31" t="s">
+      <c r="D21" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="E21" s="31" t="s">
+      <c r="E21" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="F21" s="31" t="s">
+      <c r="F21" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="G21" s="31"/>
-      <c r="H21" s="22" t="s">
+      <c r="G21" s="32"/>
+      <c r="H21" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="I21" s="34" t="s">
+      <c r="I21" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="J21" s="31"/>
+      <c r="J21" s="32"/>
     </row>
     <row r="22" ht="69.75" customHeight="1">
-      <c r="A22" s="35"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
+      <c r="A22" s="36"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
     </row>
     <row r="23" ht="69.75" customHeight="1">
-      <c r="A23" s="35"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
+      <c r="A23" s="36"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
     </row>
     <row r="24" ht="69.75" customHeight="1">
-      <c r="A24" s="35"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="35"/>
+      <c r="A24" s="36"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="36"/>
     </row>
     <row r="25" ht="69.75" customHeight="1">
-      <c r="A25" s="35"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="35"/>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
-      <c r="J25" s="35"/>
+      <c r="A25" s="36"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="36"/>
+      <c r="J25" s="36"/>
     </row>
     <row r="26" ht="69.75" customHeight="1">
-      <c r="A26" s="35"/>
-      <c r="B26" s="35"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="35"/>
-      <c r="G26" s="35"/>
-      <c r="H26" s="35"/>
-      <c r="I26" s="35"/>
-      <c r="J26" s="35"/>
+      <c r="A26" s="36"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="36"/>
+      <c r="J26" s="36"/>
     </row>
     <row r="27" ht="69.75" customHeight="1">
-      <c r="A27" s="35"/>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="35"/>
+      <c r="A27" s="36"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="36"/>
+      <c r="J27" s="36"/>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1"/>
@@ -5120,15 +5164,1019 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
+    <row r="1005" ht="15.75" customHeight="1"/>
+    <row r="1006" ht="15.75" customHeight="1"/>
+    <row r="1007" ht="15.75" customHeight="1"/>
+    <row r="1008" ht="15.75" customHeight="1"/>
+    <row r="1009" ht="15.75" customHeight="1"/>
+    <row r="1010" ht="15.75" customHeight="1"/>
+    <row r="1011" ht="15.75" customHeight="1"/>
+    <row r="1012" ht="15.75" customHeight="1"/>
+    <row r="1013" ht="15.75" customHeight="1"/>
+    <row r="1014" ht="15.75" customHeight="1"/>
+    <row r="1015" ht="15.75" customHeight="1"/>
+    <row r="1016" ht="15.75" customHeight="1"/>
+    <row r="1017" ht="15.75" customHeight="1"/>
+    <row r="1018" ht="15.75" customHeight="1"/>
+    <row r="1019" ht="15.75" customHeight="1"/>
+    <row r="1020" ht="15.75" customHeight="1"/>
+    <row r="1021" ht="15.75" customHeight="1"/>
+    <row r="1022" ht="15.75" customHeight="1"/>
+    <row r="1023" ht="15.75" customHeight="1"/>
+    <row r="1024" ht="15.75" customHeight="1"/>
+    <row r="1025" ht="15.75" customHeight="1"/>
+    <row r="1026" ht="15.75" customHeight="1"/>
+    <row r="1027" ht="15.75" customHeight="1"/>
+    <row r="1028" ht="15.75" customHeight="1"/>
+    <row r="1029" ht="15.75" customHeight="1"/>
+    <row r="1030" ht="15.75" customHeight="1"/>
+    <row r="1031" ht="15.75" customHeight="1"/>
+    <row r="1032" ht="15.75" customHeight="1"/>
+    <row r="1033" ht="15.75" customHeight="1"/>
+    <row r="1034" ht="15.75" customHeight="1"/>
+    <row r="1035" ht="15.75" customHeight="1"/>
+    <row r="1036" ht="15.75" customHeight="1"/>
+    <row r="1037" ht="15.75" customHeight="1"/>
+    <row r="1038" ht="15.75" customHeight="1"/>
+    <row r="1039" ht="15.75" customHeight="1"/>
+    <row r="1040" ht="15.75" customHeight="1"/>
+    <row r="1041" ht="15.75" customHeight="1"/>
+    <row r="1042" ht="15.75" customHeight="1"/>
+    <row r="1043" ht="15.75" customHeight="1"/>
+    <row r="1044" ht="15.75" customHeight="1"/>
+    <row r="1045" ht="15.75" customHeight="1"/>
+    <row r="1046" ht="15.75" customHeight="1"/>
+    <row r="1047" ht="15.75" customHeight="1"/>
+    <row r="1048" ht="15.75" customHeight="1"/>
+    <row r="1049" ht="15.75" customHeight="1"/>
+    <row r="1050" ht="15.75" customHeight="1"/>
+    <row r="1051" ht="15.75" customHeight="1"/>
+    <row r="1052" ht="15.75" customHeight="1"/>
+    <row r="1053" ht="15.75" customHeight="1"/>
+    <row r="1054" ht="15.75" customHeight="1"/>
+    <row r="1055" ht="15.75" customHeight="1"/>
+    <row r="1056" ht="15.75" customHeight="1"/>
+    <row r="1057" ht="15.75" customHeight="1"/>
+    <row r="1058" ht="15.75" customHeight="1"/>
+    <row r="1059" ht="15.75" customHeight="1"/>
+    <row r="1060" ht="15.75" customHeight="1"/>
+    <row r="1061" ht="15.75" customHeight="1"/>
+    <row r="1062" ht="15.75" customHeight="1"/>
+    <row r="1063" ht="15.75" customHeight="1"/>
+    <row r="1064" ht="15.75" customHeight="1"/>
+    <row r="1065" ht="15.75" customHeight="1"/>
+    <row r="1066" ht="15.75" customHeight="1"/>
+    <row r="1067" ht="15.75" customHeight="1"/>
+    <row r="1068" ht="15.75" customHeight="1"/>
+    <row r="1069" ht="15.75" customHeight="1"/>
+    <row r="1070" ht="15.75" customHeight="1"/>
+    <row r="1071" ht="15.75" customHeight="1"/>
+    <row r="1072" ht="15.75" customHeight="1"/>
+    <row r="1073" ht="15.75" customHeight="1"/>
+    <row r="1074" ht="15.75" customHeight="1"/>
+    <row r="1075" ht="15.75" customHeight="1"/>
+    <row r="1076" ht="15.75" customHeight="1"/>
+    <row r="1077" ht="15.75" customHeight="1"/>
+    <row r="1078" ht="15.75" customHeight="1"/>
+    <row r="1079" ht="15.75" customHeight="1"/>
+    <row r="1080" ht="15.75" customHeight="1"/>
+    <row r="1081" ht="15.75" customHeight="1"/>
+    <row r="1082" ht="15.75" customHeight="1"/>
+    <row r="1083" ht="15.75" customHeight="1"/>
+    <row r="1084" ht="15.75" customHeight="1"/>
+    <row r="1085" ht="15.75" customHeight="1"/>
+    <row r="1086" ht="15.75" customHeight="1"/>
+    <row r="1087" ht="15.75" customHeight="1"/>
+    <row r="1088" ht="15.75" customHeight="1"/>
+    <row r="1089" ht="15.75" customHeight="1"/>
+    <row r="1090" ht="15.75" customHeight="1"/>
+    <row r="1091" ht="15.75" customHeight="1"/>
+    <row r="1092" ht="15.75" customHeight="1"/>
+    <row r="1093" ht="15.75" customHeight="1"/>
+    <row r="1094" ht="15.75" customHeight="1"/>
+    <row r="1095" ht="15.75" customHeight="1"/>
+    <row r="1096" ht="15.75" customHeight="1"/>
+    <row r="1097" ht="15.75" customHeight="1"/>
+    <row r="1098" ht="15.75" customHeight="1"/>
+    <row r="1099" ht="15.75" customHeight="1"/>
+    <row r="1100" ht="15.75" customHeight="1"/>
+    <row r="1101" ht="15.75" customHeight="1"/>
+    <row r="1102" ht="15.75" customHeight="1"/>
+    <row r="1103" ht="15.75" customHeight="1"/>
+    <row r="1104" ht="15.75" customHeight="1"/>
+    <row r="1105" ht="15.75" customHeight="1"/>
+    <row r="1106" ht="15.75" customHeight="1"/>
+    <row r="1107" ht="15.75" customHeight="1"/>
+    <row r="1108" ht="15.75" customHeight="1"/>
+    <row r="1109" ht="15.75" customHeight="1"/>
+    <row r="1110" ht="15.75" customHeight="1"/>
+    <row r="1111" ht="15.75" customHeight="1"/>
+    <row r="1112" ht="15.75" customHeight="1"/>
+    <row r="1113" ht="15.75" customHeight="1"/>
+    <row r="1114" ht="15.75" customHeight="1"/>
+    <row r="1115" ht="15.75" customHeight="1"/>
+    <row r="1116" ht="15.75" customHeight="1"/>
+    <row r="1117" ht="15.75" customHeight="1"/>
+    <row r="1118" ht="15.75" customHeight="1"/>
+    <row r="1119" ht="15.75" customHeight="1"/>
+    <row r="1120" ht="15.75" customHeight="1"/>
+    <row r="1121" ht="15.75" customHeight="1"/>
+    <row r="1122" ht="15.75" customHeight="1"/>
+    <row r="1123" ht="15.75" customHeight="1"/>
+    <row r="1124" ht="15.75" customHeight="1"/>
+    <row r="1125" ht="15.75" customHeight="1"/>
+    <row r="1126" ht="15.75" customHeight="1"/>
+    <row r="1127" ht="15.75" customHeight="1"/>
+    <row r="1128" ht="15.75" customHeight="1"/>
+    <row r="1129" ht="15.75" customHeight="1"/>
+    <row r="1130" ht="15.75" customHeight="1"/>
+    <row r="1131" ht="15.75" customHeight="1"/>
+    <row r="1132" ht="15.75" customHeight="1"/>
+    <row r="1133" ht="15.75" customHeight="1"/>
+    <row r="1134" ht="15.75" customHeight="1"/>
+    <row r="1135" ht="15.75" customHeight="1"/>
+    <row r="1136" ht="15.75" customHeight="1"/>
+    <row r="1137" ht="15.75" customHeight="1"/>
+    <row r="1138" ht="15.75" customHeight="1"/>
+    <row r="1139" ht="15.75" customHeight="1"/>
+    <row r="1140" ht="15.75" customHeight="1"/>
+    <row r="1141" ht="15.75" customHeight="1"/>
+    <row r="1142" ht="15.75" customHeight="1"/>
+    <row r="1143" ht="15.75" customHeight="1"/>
+    <row r="1144" ht="15.75" customHeight="1"/>
+    <row r="1145" ht="15.75" customHeight="1"/>
+    <row r="1146" ht="15.75" customHeight="1"/>
+    <row r="1147" ht="15.75" customHeight="1"/>
+    <row r="1148" ht="15.75" customHeight="1"/>
+    <row r="1149" ht="15.75" customHeight="1"/>
+    <row r="1150" ht="15.75" customHeight="1"/>
+    <row r="1151" ht="15.75" customHeight="1"/>
+    <row r="1152" ht="15.75" customHeight="1"/>
+    <row r="1153" ht="15.75" customHeight="1"/>
+    <row r="1154" ht="15.75" customHeight="1"/>
+    <row r="1155" ht="15.75" customHeight="1"/>
+    <row r="1156" ht="15.75" customHeight="1"/>
+    <row r="1157" ht="15.75" customHeight="1"/>
+    <row r="1158" ht="15.75" customHeight="1"/>
+    <row r="1159" ht="15.75" customHeight="1"/>
+    <row r="1160" ht="15.75" customHeight="1"/>
+    <row r="1161" ht="15.75" customHeight="1"/>
+    <row r="1162" ht="15.75" customHeight="1"/>
+    <row r="1163" ht="15.75" customHeight="1"/>
+    <row r="1164" ht="15.75" customHeight="1"/>
+    <row r="1165" ht="15.75" customHeight="1"/>
+    <row r="1166" ht="15.75" customHeight="1"/>
+    <row r="1167" ht="15.75" customHeight="1"/>
+    <row r="1168" ht="15.75" customHeight="1"/>
+    <row r="1169" ht="15.75" customHeight="1"/>
+    <row r="1170" ht="15.75" customHeight="1"/>
+    <row r="1171" ht="15.75" customHeight="1"/>
+    <row r="1172" ht="15.75" customHeight="1"/>
+    <row r="1173" ht="15.75" customHeight="1"/>
+    <row r="1174" ht="15.75" customHeight="1"/>
+    <row r="1175" ht="15.75" customHeight="1"/>
+    <row r="1176" ht="15.75" customHeight="1"/>
+    <row r="1177" ht="15.75" customHeight="1"/>
+    <row r="1178" ht="15.75" customHeight="1"/>
+    <row r="1179" ht="15.75" customHeight="1"/>
+    <row r="1180" ht="15.75" customHeight="1"/>
+    <row r="1181" ht="15.75" customHeight="1"/>
+    <row r="1182" ht="15.75" customHeight="1"/>
+    <row r="1183" ht="15.75" customHeight="1"/>
+    <row r="1184" ht="15.75" customHeight="1"/>
+    <row r="1185" ht="15.75" customHeight="1"/>
+    <row r="1186" ht="15.75" customHeight="1"/>
+    <row r="1187" ht="15.75" customHeight="1"/>
+    <row r="1188" ht="15.75" customHeight="1"/>
+    <row r="1189" ht="15.75" customHeight="1"/>
+    <row r="1190" ht="15.75" customHeight="1"/>
+    <row r="1191" ht="15.75" customHeight="1"/>
+    <row r="1192" ht="15.75" customHeight="1"/>
+    <row r="1193" ht="15.75" customHeight="1"/>
+    <row r="1194" ht="15.75" customHeight="1"/>
+    <row r="1195" ht="15.75" customHeight="1"/>
+    <row r="1196" ht="15.75" customHeight="1"/>
+    <row r="1197" ht="15.75" customHeight="1"/>
+    <row r="1198" ht="15.75" customHeight="1"/>
+    <row r="1199" ht="15.75" customHeight="1"/>
+    <row r="1200" ht="15.75" customHeight="1"/>
+    <row r="1201" ht="15.75" customHeight="1"/>
+    <row r="1202" ht="15.75" customHeight="1"/>
+    <row r="1203" ht="15.75" customHeight="1"/>
+    <row r="1204" ht="15.75" customHeight="1"/>
+    <row r="1205" ht="15.75" customHeight="1"/>
+    <row r="1206" ht="15.75" customHeight="1"/>
+    <row r="1207" ht="15.75" customHeight="1"/>
+    <row r="1208" ht="15.75" customHeight="1"/>
+    <row r="1209" ht="15.75" customHeight="1"/>
+    <row r="1210" ht="15.75" customHeight="1"/>
+    <row r="1211" ht="15.75" customHeight="1"/>
+    <row r="1212" ht="15.75" customHeight="1"/>
+    <row r="1213" ht="15.75" customHeight="1"/>
+    <row r="1214" ht="15.75" customHeight="1"/>
+    <row r="1215" ht="15.75" customHeight="1"/>
+    <row r="1216" ht="15.75" customHeight="1"/>
+    <row r="1217" ht="15.75" customHeight="1"/>
+    <row r="1218" ht="15.75" customHeight="1"/>
+    <row r="1219" ht="15.75" customHeight="1"/>
+    <row r="1220" ht="15.75" customHeight="1"/>
+    <row r="1221" ht="15.75" customHeight="1"/>
+    <row r="1222" ht="15.75" customHeight="1"/>
+    <row r="1223" ht="15.75" customHeight="1"/>
+    <row r="1224" ht="15.75" customHeight="1"/>
+    <row r="1225" ht="15.75" customHeight="1"/>
+    <row r="1226" ht="15.75" customHeight="1"/>
+    <row r="1227" ht="15.75" customHeight="1"/>
+    <row r="1228" ht="15.75" customHeight="1"/>
+    <row r="1229" ht="15.75" customHeight="1"/>
+    <row r="1230" ht="15.75" customHeight="1"/>
+    <row r="1231" ht="15.75" customHeight="1"/>
+    <row r="1232" ht="15.75" customHeight="1"/>
+    <row r="1233" ht="15.75" customHeight="1"/>
+    <row r="1234" ht="15.75" customHeight="1"/>
+    <row r="1235" ht="15.75" customHeight="1"/>
+    <row r="1236" ht="15.75" customHeight="1"/>
+    <row r="1237" ht="15.75" customHeight="1"/>
+    <row r="1238" ht="15.75" customHeight="1"/>
+    <row r="1239" ht="15.75" customHeight="1"/>
+    <row r="1240" ht="15.75" customHeight="1"/>
+    <row r="1241" ht="15.75" customHeight="1"/>
+    <row r="1242" ht="15.75" customHeight="1"/>
+    <row r="1243" ht="15.75" customHeight="1"/>
+    <row r="1244" ht="15.75" customHeight="1"/>
+    <row r="1245" ht="15.75" customHeight="1"/>
+    <row r="1246" ht="15.75" customHeight="1"/>
+    <row r="1247" ht="15.75" customHeight="1"/>
+    <row r="1248" ht="15.75" customHeight="1"/>
+    <row r="1249" ht="15.75" customHeight="1"/>
+    <row r="1250" ht="15.75" customHeight="1"/>
+    <row r="1251" ht="15.75" customHeight="1"/>
+    <row r="1252" ht="15.75" customHeight="1"/>
+    <row r="1253" ht="15.75" customHeight="1"/>
+    <row r="1254" ht="15.75" customHeight="1"/>
+    <row r="1255" ht="15.75" customHeight="1"/>
+    <row r="1256" ht="15.75" customHeight="1"/>
+    <row r="1257" ht="15.75" customHeight="1"/>
+    <row r="1258" ht="15.75" customHeight="1"/>
+    <row r="1259" ht="15.75" customHeight="1"/>
+    <row r="1260" ht="15.75" customHeight="1"/>
+    <row r="1261" ht="15.75" customHeight="1"/>
+    <row r="1262" ht="15.75" customHeight="1"/>
+    <row r="1263" ht="15.75" customHeight="1"/>
+    <row r="1264" ht="15.75" customHeight="1"/>
+    <row r="1265" ht="15.75" customHeight="1"/>
+    <row r="1266" ht="15.75" customHeight="1"/>
+    <row r="1267" ht="15.75" customHeight="1"/>
+    <row r="1268" ht="15.75" customHeight="1"/>
+    <row r="1269" ht="15.75" customHeight="1"/>
+    <row r="1270" ht="15.75" customHeight="1"/>
+    <row r="1271" ht="15.75" customHeight="1"/>
+    <row r="1272" ht="15.75" customHeight="1"/>
+    <row r="1273" ht="15.75" customHeight="1"/>
+    <row r="1274" ht="15.75" customHeight="1"/>
+    <row r="1275" ht="15.75" customHeight="1"/>
+    <row r="1276" ht="15.75" customHeight="1"/>
+    <row r="1277" ht="15.75" customHeight="1"/>
+    <row r="1278" ht="15.75" customHeight="1"/>
+    <row r="1279" ht="15.75" customHeight="1"/>
+    <row r="1280" ht="15.75" customHeight="1"/>
+    <row r="1281" ht="15.75" customHeight="1"/>
+    <row r="1282" ht="15.75" customHeight="1"/>
+    <row r="1283" ht="15.75" customHeight="1"/>
+    <row r="1284" ht="15.75" customHeight="1"/>
+    <row r="1285" ht="15.75" customHeight="1"/>
+    <row r="1286" ht="15.75" customHeight="1"/>
+    <row r="1287" ht="15.75" customHeight="1"/>
+    <row r="1288" ht="15.75" customHeight="1"/>
+    <row r="1289" ht="15.75" customHeight="1"/>
+    <row r="1290" ht="15.75" customHeight="1"/>
+    <row r="1291" ht="15.75" customHeight="1"/>
+    <row r="1292" ht="15.75" customHeight="1"/>
+    <row r="1293" ht="15.75" customHeight="1"/>
+    <row r="1294" ht="15.75" customHeight="1"/>
+    <row r="1295" ht="15.75" customHeight="1"/>
+    <row r="1296" ht="15.75" customHeight="1"/>
+    <row r="1297" ht="15.75" customHeight="1"/>
+    <row r="1298" ht="15.75" customHeight="1"/>
+    <row r="1299" ht="15.75" customHeight="1"/>
+    <row r="1300" ht="15.75" customHeight="1"/>
+    <row r="1301" ht="15.75" customHeight="1"/>
+    <row r="1302" ht="15.75" customHeight="1"/>
+    <row r="1303" ht="15.75" customHeight="1"/>
+    <row r="1304" ht="15.75" customHeight="1"/>
+    <row r="1305" ht="15.75" customHeight="1"/>
+    <row r="1306" ht="15.75" customHeight="1"/>
+    <row r="1307" ht="15.75" customHeight="1"/>
+    <row r="1308" ht="15.75" customHeight="1"/>
+    <row r="1309" ht="15.75" customHeight="1"/>
+    <row r="1310" ht="15.75" customHeight="1"/>
+    <row r="1311" ht="15.75" customHeight="1"/>
+    <row r="1312" ht="15.75" customHeight="1"/>
+    <row r="1313" ht="15.75" customHeight="1"/>
+    <row r="1314" ht="15.75" customHeight="1"/>
+    <row r="1315" ht="15.75" customHeight="1"/>
+    <row r="1316" ht="15.75" customHeight="1"/>
+    <row r="1317" ht="15.75" customHeight="1"/>
+    <row r="1318" ht="15.75" customHeight="1"/>
+    <row r="1319" ht="15.75" customHeight="1"/>
+    <row r="1320" ht="15.75" customHeight="1"/>
+    <row r="1321" ht="15.75" customHeight="1"/>
+    <row r="1322" ht="15.75" customHeight="1"/>
+    <row r="1323" ht="15.75" customHeight="1"/>
+    <row r="1324" ht="15.75" customHeight="1"/>
+    <row r="1325" ht="15.75" customHeight="1"/>
+    <row r="1326" ht="15.75" customHeight="1"/>
+    <row r="1327" ht="15.75" customHeight="1"/>
+    <row r="1328" ht="15.75" customHeight="1"/>
+    <row r="1329" ht="15.75" customHeight="1"/>
+    <row r="1330" ht="15.75" customHeight="1"/>
+    <row r="1331" ht="15.75" customHeight="1"/>
+    <row r="1332" ht="15.75" customHeight="1"/>
+    <row r="1333" ht="15.75" customHeight="1"/>
+    <row r="1334" ht="15.75" customHeight="1"/>
+    <row r="1335" ht="15.75" customHeight="1"/>
+    <row r="1336" ht="15.75" customHeight="1"/>
+    <row r="1337" ht="15.75" customHeight="1"/>
+    <row r="1338" ht="15.75" customHeight="1"/>
+    <row r="1339" ht="15.75" customHeight="1"/>
+    <row r="1340" ht="15.75" customHeight="1"/>
+    <row r="1341" ht="15.75" customHeight="1"/>
+    <row r="1342" ht="15.75" customHeight="1"/>
+    <row r="1343" ht="15.75" customHeight="1"/>
+    <row r="1344" ht="15.75" customHeight="1"/>
+    <row r="1345" ht="15.75" customHeight="1"/>
+    <row r="1346" ht="15.75" customHeight="1"/>
+    <row r="1347" ht="15.75" customHeight="1"/>
+    <row r="1348" ht="15.75" customHeight="1"/>
+    <row r="1349" ht="15.75" customHeight="1"/>
+    <row r="1350" ht="15.75" customHeight="1"/>
+    <row r="1351" ht="15.75" customHeight="1"/>
+    <row r="1352" ht="15.75" customHeight="1"/>
+    <row r="1353" ht="15.75" customHeight="1"/>
+    <row r="1354" ht="15.75" customHeight="1"/>
+    <row r="1355" ht="15.75" customHeight="1"/>
+    <row r="1356" ht="15.75" customHeight="1"/>
+    <row r="1357" ht="15.75" customHeight="1"/>
+    <row r="1358" ht="15.75" customHeight="1"/>
+    <row r="1359" ht="15.75" customHeight="1"/>
+    <row r="1360" ht="15.75" customHeight="1"/>
+    <row r="1361" ht="15.75" customHeight="1"/>
+    <row r="1362" ht="15.75" customHeight="1"/>
+    <row r="1363" ht="15.75" customHeight="1"/>
+    <row r="1364" ht="15.75" customHeight="1"/>
+    <row r="1365" ht="15.75" customHeight="1"/>
+    <row r="1366" ht="15.75" customHeight="1"/>
+    <row r="1367" ht="15.75" customHeight="1"/>
+    <row r="1368" ht="15.75" customHeight="1"/>
+    <row r="1369" ht="15.75" customHeight="1"/>
+    <row r="1370" ht="15.75" customHeight="1"/>
+    <row r="1371" ht="15.75" customHeight="1"/>
+    <row r="1372" ht="15.75" customHeight="1"/>
+    <row r="1373" ht="15.75" customHeight="1"/>
+    <row r="1374" ht="15.75" customHeight="1"/>
+    <row r="1375" ht="15.75" customHeight="1"/>
+    <row r="1376" ht="15.75" customHeight="1"/>
+    <row r="1377" ht="15.75" customHeight="1"/>
+    <row r="1378" ht="15.75" customHeight="1"/>
+    <row r="1379" ht="15.75" customHeight="1"/>
+    <row r="1380" ht="15.75" customHeight="1"/>
+    <row r="1381" ht="15.75" customHeight="1"/>
+    <row r="1382" ht="15.75" customHeight="1"/>
+    <row r="1383" ht="15.75" customHeight="1"/>
+    <row r="1384" ht="15.75" customHeight="1"/>
+    <row r="1385" ht="15.75" customHeight="1"/>
+    <row r="1386" ht="15.75" customHeight="1"/>
+    <row r="1387" ht="15.75" customHeight="1"/>
+    <row r="1388" ht="15.75" customHeight="1"/>
+    <row r="1389" ht="15.75" customHeight="1"/>
+    <row r="1390" ht="15.75" customHeight="1"/>
+    <row r="1391" ht="15.75" customHeight="1"/>
+    <row r="1392" ht="15.75" customHeight="1"/>
+    <row r="1393" ht="15.75" customHeight="1"/>
+    <row r="1394" ht="15.75" customHeight="1"/>
+    <row r="1395" ht="15.75" customHeight="1"/>
+    <row r="1396" ht="15.75" customHeight="1"/>
+    <row r="1397" ht="15.75" customHeight="1"/>
+    <row r="1398" ht="15.75" customHeight="1"/>
+    <row r="1399" ht="15.75" customHeight="1"/>
+    <row r="1400" ht="15.75" customHeight="1"/>
+    <row r="1401" ht="15.75" customHeight="1"/>
+    <row r="1402" ht="15.75" customHeight="1"/>
+    <row r="1403" ht="15.75" customHeight="1"/>
+    <row r="1404" ht="15.75" customHeight="1"/>
+    <row r="1405" ht="15.75" customHeight="1"/>
+    <row r="1406" ht="15.75" customHeight="1"/>
+    <row r="1407" ht="15.75" customHeight="1"/>
+    <row r="1408" ht="15.75" customHeight="1"/>
+    <row r="1409" ht="15.75" customHeight="1"/>
+    <row r="1410" ht="15.75" customHeight="1"/>
+    <row r="1411" ht="15.75" customHeight="1"/>
+    <row r="1412" ht="15.75" customHeight="1"/>
+    <row r="1413" ht="15.75" customHeight="1"/>
+    <row r="1414" ht="15.75" customHeight="1"/>
+    <row r="1415" ht="15.75" customHeight="1"/>
+    <row r="1416" ht="15.75" customHeight="1"/>
+    <row r="1417" ht="15.75" customHeight="1"/>
+    <row r="1418" ht="15.75" customHeight="1"/>
+    <row r="1419" ht="15.75" customHeight="1"/>
+    <row r="1420" ht="15.75" customHeight="1"/>
+    <row r="1421" ht="15.75" customHeight="1"/>
+    <row r="1422" ht="15.75" customHeight="1"/>
+    <row r="1423" ht="15.75" customHeight="1"/>
+    <row r="1424" ht="15.75" customHeight="1"/>
+    <row r="1425" ht="15.75" customHeight="1"/>
+    <row r="1426" ht="15.75" customHeight="1"/>
+    <row r="1427" ht="15.75" customHeight="1"/>
+    <row r="1428" ht="15.75" customHeight="1"/>
+    <row r="1429" ht="15.75" customHeight="1"/>
+    <row r="1430" ht="15.75" customHeight="1"/>
+    <row r="1431" ht="15.75" customHeight="1"/>
+    <row r="1432" ht="15.75" customHeight="1"/>
+    <row r="1433" ht="15.75" customHeight="1"/>
+    <row r="1434" ht="15.75" customHeight="1"/>
+    <row r="1435" ht="15.75" customHeight="1"/>
+    <row r="1436" ht="15.75" customHeight="1"/>
+    <row r="1437" ht="15.75" customHeight="1"/>
+    <row r="1438" ht="15.75" customHeight="1"/>
+    <row r="1439" ht="15.75" customHeight="1"/>
+    <row r="1440" ht="15.75" customHeight="1"/>
+    <row r="1441" ht="15.75" customHeight="1"/>
+    <row r="1442" ht="15.75" customHeight="1"/>
+    <row r="1443" ht="15.75" customHeight="1"/>
+    <row r="1444" ht="15.75" customHeight="1"/>
+    <row r="1445" ht="15.75" customHeight="1"/>
+    <row r="1446" ht="15.75" customHeight="1"/>
+    <row r="1447" ht="15.75" customHeight="1"/>
+    <row r="1448" ht="15.75" customHeight="1"/>
+    <row r="1449" ht="15.75" customHeight="1"/>
+    <row r="1450" ht="15.75" customHeight="1"/>
+    <row r="1451" ht="15.75" customHeight="1"/>
+    <row r="1452" ht="15.75" customHeight="1"/>
+    <row r="1453" ht="15.75" customHeight="1"/>
+    <row r="1454" ht="15.75" customHeight="1"/>
+    <row r="1455" ht="15.75" customHeight="1"/>
+    <row r="1456" ht="15.75" customHeight="1"/>
+    <row r="1457" ht="15.75" customHeight="1"/>
+    <row r="1458" ht="15.75" customHeight="1"/>
+    <row r="1459" ht="15.75" customHeight="1"/>
+    <row r="1460" ht="15.75" customHeight="1"/>
+    <row r="1461" ht="15.75" customHeight="1"/>
+    <row r="1462" ht="15.75" customHeight="1"/>
+    <row r="1463" ht="15.75" customHeight="1"/>
+    <row r="1464" ht="15.75" customHeight="1"/>
+    <row r="1465" ht="15.75" customHeight="1"/>
+    <row r="1466" ht="15.75" customHeight="1"/>
+    <row r="1467" ht="15.75" customHeight="1"/>
+    <row r="1468" ht="15.75" customHeight="1"/>
+    <row r="1469" ht="15.75" customHeight="1"/>
+    <row r="1470" ht="15.75" customHeight="1"/>
+    <row r="1471" ht="15.75" customHeight="1"/>
+    <row r="1472" ht="15.75" customHeight="1"/>
+    <row r="1473" ht="15.75" customHeight="1"/>
+    <row r="1474" ht="15.75" customHeight="1"/>
+    <row r="1475" ht="15.75" customHeight="1"/>
+    <row r="1476" ht="15.75" customHeight="1"/>
+    <row r="1477" ht="15.75" customHeight="1"/>
+    <row r="1478" ht="15.75" customHeight="1"/>
+    <row r="1479" ht="15.75" customHeight="1"/>
+    <row r="1480" ht="15.75" customHeight="1"/>
+    <row r="1481" ht="15.75" customHeight="1"/>
+    <row r="1482" ht="15.75" customHeight="1"/>
+    <row r="1483" ht="15.75" customHeight="1"/>
+    <row r="1484" ht="15.75" customHeight="1"/>
+    <row r="1485" ht="15.75" customHeight="1"/>
+    <row r="1486" ht="15.75" customHeight="1"/>
+    <row r="1487" ht="15.75" customHeight="1"/>
+    <row r="1488" ht="15.75" customHeight="1"/>
+    <row r="1489" ht="15.75" customHeight="1"/>
+    <row r="1490" ht="15.75" customHeight="1"/>
+    <row r="1491" ht="15.75" customHeight="1"/>
+    <row r="1492" ht="15.75" customHeight="1"/>
+    <row r="1493" ht="15.75" customHeight="1"/>
+    <row r="1494" ht="15.75" customHeight="1"/>
+    <row r="1495" ht="15.75" customHeight="1"/>
+    <row r="1496" ht="15.75" customHeight="1"/>
+    <row r="1497" ht="15.75" customHeight="1"/>
+    <row r="1498" ht="15.75" customHeight="1"/>
+    <row r="1499" ht="15.75" customHeight="1"/>
+    <row r="1500" ht="15.75" customHeight="1"/>
+    <row r="1501" ht="15.75" customHeight="1"/>
+    <row r="1502" ht="15.75" customHeight="1"/>
+    <row r="1503" ht="15.75" customHeight="1"/>
+    <row r="1504" ht="15.75" customHeight="1"/>
+    <row r="1505" ht="15.75" customHeight="1"/>
+    <row r="1506" ht="15.75" customHeight="1"/>
+    <row r="1507" ht="15.75" customHeight="1"/>
+    <row r="1508" ht="15.75" customHeight="1"/>
+    <row r="1509" ht="15.75" customHeight="1"/>
+    <row r="1510" ht="15.75" customHeight="1"/>
+    <row r="1511" ht="15.75" customHeight="1"/>
+    <row r="1512" ht="15.75" customHeight="1"/>
+    <row r="1513" ht="15.75" customHeight="1"/>
+    <row r="1514" ht="15.75" customHeight="1"/>
+    <row r="1515" ht="15.75" customHeight="1"/>
+    <row r="1516" ht="15.75" customHeight="1"/>
+    <row r="1517" ht="15.75" customHeight="1"/>
+    <row r="1518" ht="15.75" customHeight="1"/>
+    <row r="1519" ht="15.75" customHeight="1"/>
+    <row r="1520" ht="15.75" customHeight="1"/>
+    <row r="1521" ht="15.75" customHeight="1"/>
+    <row r="1522" ht="15.75" customHeight="1"/>
+    <row r="1523" ht="15.75" customHeight="1"/>
+    <row r="1524" ht="15.75" customHeight="1"/>
+    <row r="1525" ht="15.75" customHeight="1"/>
+    <row r="1526" ht="15.75" customHeight="1"/>
+    <row r="1527" ht="15.75" customHeight="1"/>
+    <row r="1528" ht="15.75" customHeight="1"/>
+    <row r="1529" ht="15.75" customHeight="1"/>
+    <row r="1530" ht="15.75" customHeight="1"/>
+    <row r="1531" ht="15.75" customHeight="1"/>
+    <row r="1532" ht="15.75" customHeight="1"/>
+    <row r="1533" ht="15.75" customHeight="1"/>
+    <row r="1534" ht="15.75" customHeight="1"/>
+    <row r="1535" ht="15.75" customHeight="1"/>
+    <row r="1536" ht="15.75" customHeight="1"/>
+    <row r="1537" ht="15.75" customHeight="1"/>
+    <row r="1538" ht="15.75" customHeight="1"/>
+    <row r="1539" ht="15.75" customHeight="1"/>
+    <row r="1540" ht="15.75" customHeight="1"/>
+    <row r="1541" ht="15.75" customHeight="1"/>
+    <row r="1542" ht="15.75" customHeight="1"/>
+    <row r="1543" ht="15.75" customHeight="1"/>
+    <row r="1544" ht="15.75" customHeight="1"/>
+    <row r="1545" ht="15.75" customHeight="1"/>
+    <row r="1546" ht="15.75" customHeight="1"/>
+    <row r="1547" ht="15.75" customHeight="1"/>
+    <row r="1548" ht="15.75" customHeight="1"/>
+    <row r="1549" ht="15.75" customHeight="1"/>
+    <row r="1550" ht="15.75" customHeight="1"/>
+    <row r="1551" ht="15.75" customHeight="1"/>
+    <row r="1552" ht="15.75" customHeight="1"/>
+    <row r="1553" ht="15.75" customHeight="1"/>
+    <row r="1554" ht="15.75" customHeight="1"/>
+    <row r="1555" ht="15.75" customHeight="1"/>
+    <row r="1556" ht="15.75" customHeight="1"/>
+    <row r="1557" ht="15.75" customHeight="1"/>
+    <row r="1558" ht="15.75" customHeight="1"/>
+    <row r="1559" ht="15.75" customHeight="1"/>
+    <row r="1560" ht="15.75" customHeight="1"/>
+    <row r="1561" ht="15.75" customHeight="1"/>
+    <row r="1562" ht="15.75" customHeight="1"/>
+    <row r="1563" ht="15.75" customHeight="1"/>
+    <row r="1564" ht="15.75" customHeight="1"/>
+    <row r="1565" ht="15.75" customHeight="1"/>
+    <row r="1566" ht="15.75" customHeight="1"/>
+    <row r="1567" ht="15.75" customHeight="1"/>
+    <row r="1568" ht="15.75" customHeight="1"/>
+    <row r="1569" ht="15.75" customHeight="1"/>
+    <row r="1570" ht="15.75" customHeight="1"/>
+    <row r="1571" ht="15.75" customHeight="1"/>
+    <row r="1572" ht="15.75" customHeight="1"/>
+    <row r="1573" ht="15.75" customHeight="1"/>
+    <row r="1574" ht="15.75" customHeight="1"/>
+    <row r="1575" ht="15.75" customHeight="1"/>
+    <row r="1576" ht="15.75" customHeight="1"/>
+    <row r="1577" ht="15.75" customHeight="1"/>
+    <row r="1578" ht="15.75" customHeight="1"/>
+    <row r="1579" ht="15.75" customHeight="1"/>
+    <row r="1580" ht="15.75" customHeight="1"/>
+    <row r="1581" ht="15.75" customHeight="1"/>
+    <row r="1582" ht="15.75" customHeight="1"/>
+    <row r="1583" ht="15.75" customHeight="1"/>
+    <row r="1584" ht="15.75" customHeight="1"/>
+    <row r="1585" ht="15.75" customHeight="1"/>
+    <row r="1586" ht="15.75" customHeight="1"/>
+    <row r="1587" ht="15.75" customHeight="1"/>
+    <row r="1588" ht="15.75" customHeight="1"/>
+    <row r="1589" ht="15.75" customHeight="1"/>
+    <row r="1590" ht="15.75" customHeight="1"/>
+    <row r="1591" ht="15.75" customHeight="1"/>
+    <row r="1592" ht="15.75" customHeight="1"/>
+    <row r="1593" ht="15.75" customHeight="1"/>
+    <row r="1594" ht="15.75" customHeight="1"/>
+    <row r="1595" ht="15.75" customHeight="1"/>
+    <row r="1596" ht="15.75" customHeight="1"/>
+    <row r="1597" ht="15.75" customHeight="1"/>
+    <row r="1598" ht="15.75" customHeight="1"/>
+    <row r="1599" ht="15.75" customHeight="1"/>
+    <row r="1600" ht="15.75" customHeight="1"/>
+    <row r="1601" ht="15.75" customHeight="1"/>
+    <row r="1602" ht="15.75" customHeight="1"/>
+    <row r="1603" ht="15.75" customHeight="1"/>
+    <row r="1604" ht="15.75" customHeight="1"/>
+    <row r="1605" ht="15.75" customHeight="1"/>
+    <row r="1606" ht="15.75" customHeight="1"/>
+    <row r="1607" ht="15.75" customHeight="1"/>
+    <row r="1608" ht="15.75" customHeight="1"/>
+    <row r="1609" ht="15.75" customHeight="1"/>
+    <row r="1610" ht="15.75" customHeight="1"/>
+    <row r="1611" ht="15.75" customHeight="1"/>
+    <row r="1612" ht="15.75" customHeight="1"/>
+    <row r="1613" ht="15.75" customHeight="1"/>
+    <row r="1614" ht="15.75" customHeight="1"/>
+    <row r="1615" ht="15.75" customHeight="1"/>
+    <row r="1616" ht="15.75" customHeight="1"/>
+    <row r="1617" ht="15.75" customHeight="1"/>
+    <row r="1618" ht="15.75" customHeight="1"/>
+    <row r="1619" ht="15.75" customHeight="1"/>
+    <row r="1620" ht="15.75" customHeight="1"/>
+    <row r="1621" ht="15.75" customHeight="1"/>
+    <row r="1622" ht="15.75" customHeight="1"/>
+    <row r="1623" ht="15.75" customHeight="1"/>
+    <row r="1624" ht="15.75" customHeight="1"/>
+    <row r="1625" ht="15.75" customHeight="1"/>
+    <row r="1626" ht="15.75" customHeight="1"/>
+    <row r="1627" ht="15.75" customHeight="1"/>
+    <row r="1628" ht="15.75" customHeight="1"/>
+    <row r="1629" ht="15.75" customHeight="1"/>
+    <row r="1630" ht="15.75" customHeight="1"/>
+    <row r="1631" ht="15.75" customHeight="1"/>
+    <row r="1632" ht="15.75" customHeight="1"/>
+    <row r="1633" ht="15.75" customHeight="1"/>
+    <row r="1634" ht="15.75" customHeight="1"/>
+    <row r="1635" ht="15.75" customHeight="1"/>
+    <row r="1636" ht="15.75" customHeight="1"/>
+    <row r="1637" ht="15.75" customHeight="1"/>
+    <row r="1638" ht="15.75" customHeight="1"/>
+    <row r="1639" ht="15.75" customHeight="1"/>
+    <row r="1640" ht="15.75" customHeight="1"/>
+    <row r="1641" ht="15.75" customHeight="1"/>
+    <row r="1642" ht="15.75" customHeight="1"/>
+    <row r="1643" ht="15.75" customHeight="1"/>
+    <row r="1644" ht="15.75" customHeight="1"/>
+    <row r="1645" ht="15.75" customHeight="1"/>
+    <row r="1646" ht="15.75" customHeight="1"/>
+    <row r="1647" ht="15.75" customHeight="1"/>
+    <row r="1648" ht="15.75" customHeight="1"/>
+    <row r="1649" ht="15.75" customHeight="1"/>
+    <row r="1650" ht="15.75" customHeight="1"/>
+    <row r="1651" ht="15.75" customHeight="1"/>
+    <row r="1652" ht="15.75" customHeight="1"/>
+    <row r="1653" ht="15.75" customHeight="1"/>
+    <row r="1654" ht="15.75" customHeight="1"/>
+    <row r="1655" ht="15.75" customHeight="1"/>
+    <row r="1656" ht="15.75" customHeight="1"/>
+    <row r="1657" ht="15.75" customHeight="1"/>
+    <row r="1658" ht="15.75" customHeight="1"/>
+    <row r="1659" ht="15.75" customHeight="1"/>
+    <row r="1660" ht="15.75" customHeight="1"/>
+    <row r="1661" ht="15.75" customHeight="1"/>
+    <row r="1662" ht="15.75" customHeight="1"/>
+    <row r="1663" ht="15.75" customHeight="1"/>
+    <row r="1664" ht="15.75" customHeight="1"/>
+    <row r="1665" ht="15.75" customHeight="1"/>
+    <row r="1666" ht="15.75" customHeight="1"/>
+    <row r="1667" ht="15.75" customHeight="1"/>
+    <row r="1668" ht="15.75" customHeight="1"/>
+    <row r="1669" ht="15.75" customHeight="1"/>
+    <row r="1670" ht="15.75" customHeight="1"/>
+    <row r="1671" ht="15.75" customHeight="1"/>
+    <row r="1672" ht="15.75" customHeight="1"/>
+    <row r="1673" ht="15.75" customHeight="1"/>
+    <row r="1674" ht="15.75" customHeight="1"/>
+    <row r="1675" ht="15.75" customHeight="1"/>
+    <row r="1676" ht="15.75" customHeight="1"/>
+    <row r="1677" ht="15.75" customHeight="1"/>
+    <row r="1678" ht="15.75" customHeight="1"/>
+    <row r="1679" ht="15.75" customHeight="1"/>
+    <row r="1680" ht="15.75" customHeight="1"/>
+    <row r="1681" ht="15.75" customHeight="1"/>
+    <row r="1682" ht="15.75" customHeight="1"/>
+    <row r="1683" ht="15.75" customHeight="1"/>
+    <row r="1684" ht="15.75" customHeight="1"/>
+    <row r="1685" ht="15.75" customHeight="1"/>
+    <row r="1686" ht="15.75" customHeight="1"/>
+    <row r="1687" ht="15.75" customHeight="1"/>
+    <row r="1688" ht="15.75" customHeight="1"/>
+    <row r="1689" ht="15.75" customHeight="1"/>
+    <row r="1690" ht="15.75" customHeight="1"/>
+    <row r="1691" ht="15.75" customHeight="1"/>
+    <row r="1692" ht="15.75" customHeight="1"/>
+    <row r="1693" ht="15.75" customHeight="1"/>
+    <row r="1694" ht="15.75" customHeight="1"/>
+    <row r="1695" ht="15.75" customHeight="1"/>
+    <row r="1696" ht="15.75" customHeight="1"/>
+    <row r="1697" ht="15.75" customHeight="1"/>
+    <row r="1698" ht="15.75" customHeight="1"/>
+    <row r="1699" ht="15.75" customHeight="1"/>
+    <row r="1700" ht="15.75" customHeight="1"/>
+    <row r="1701" ht="15.75" customHeight="1"/>
+    <row r="1702" ht="15.75" customHeight="1"/>
+    <row r="1703" ht="15.75" customHeight="1"/>
+    <row r="1704" ht="15.75" customHeight="1"/>
+    <row r="1705" ht="15.75" customHeight="1"/>
+    <row r="1706" ht="15.75" customHeight="1"/>
+    <row r="1707" ht="15.75" customHeight="1"/>
+    <row r="1708" ht="15.75" customHeight="1"/>
+    <row r="1709" ht="15.75" customHeight="1"/>
+    <row r="1710" ht="15.75" customHeight="1"/>
+    <row r="1711" ht="15.75" customHeight="1"/>
+    <row r="1712" ht="15.75" customHeight="1"/>
+    <row r="1713" ht="15.75" customHeight="1"/>
+    <row r="1714" ht="15.75" customHeight="1"/>
+    <row r="1715" ht="15.75" customHeight="1"/>
+    <row r="1716" ht="15.75" customHeight="1"/>
+    <row r="1717" ht="15.75" customHeight="1"/>
+    <row r="1718" ht="15.75" customHeight="1"/>
+    <row r="1719" ht="15.75" customHeight="1"/>
+    <row r="1720" ht="15.75" customHeight="1"/>
+    <row r="1721" ht="15.75" customHeight="1"/>
+    <row r="1722" ht="15.75" customHeight="1"/>
+    <row r="1723" ht="15.75" customHeight="1"/>
+    <row r="1724" ht="15.75" customHeight="1"/>
+    <row r="1725" ht="15.75" customHeight="1"/>
+    <row r="1726" ht="15.75" customHeight="1"/>
+    <row r="1727" ht="15.75" customHeight="1"/>
+    <row r="1728" ht="15.75" customHeight="1"/>
+    <row r="1729" ht="15.75" customHeight="1"/>
+    <row r="1730" ht="15.75" customHeight="1"/>
+    <row r="1731" ht="15.75" customHeight="1"/>
+    <row r="1732" ht="15.75" customHeight="1"/>
+    <row r="1733" ht="15.75" customHeight="1"/>
+    <row r="1734" ht="15.75" customHeight="1"/>
+    <row r="1735" ht="15.75" customHeight="1"/>
+    <row r="1736" ht="15.75" customHeight="1"/>
+    <row r="1737" ht="15.75" customHeight="1"/>
+    <row r="1738" ht="15.75" customHeight="1"/>
+    <row r="1739" ht="15.75" customHeight="1"/>
+    <row r="1740" ht="15.75" customHeight="1"/>
+    <row r="1741" ht="15.75" customHeight="1"/>
+    <row r="1742" ht="15.75" customHeight="1"/>
+    <row r="1743" ht="15.75" customHeight="1"/>
+    <row r="1744" ht="15.75" customHeight="1"/>
+    <row r="1745" ht="15.75" customHeight="1"/>
+    <row r="1746" ht="15.75" customHeight="1"/>
+    <row r="1747" ht="15.75" customHeight="1"/>
+    <row r="1748" ht="15.75" customHeight="1"/>
+    <row r="1749" ht="15.75" customHeight="1"/>
+    <row r="1750" ht="15.75" customHeight="1"/>
+    <row r="1751" ht="15.75" customHeight="1"/>
+    <row r="1752" ht="15.75" customHeight="1"/>
+    <row r="1753" ht="15.75" customHeight="1"/>
+    <row r="1754" ht="15.75" customHeight="1"/>
+    <row r="1755" ht="15.75" customHeight="1"/>
+    <row r="1756" ht="15.75" customHeight="1"/>
+    <row r="1757" ht="15.75" customHeight="1"/>
+    <row r="1758" ht="15.75" customHeight="1"/>
+    <row r="1759" ht="15.75" customHeight="1"/>
+    <row r="1760" ht="15.75" customHeight="1"/>
+    <row r="1761" ht="15.75" customHeight="1"/>
+    <row r="1762" ht="15.75" customHeight="1"/>
+    <row r="1763" ht="15.75" customHeight="1"/>
+    <row r="1764" ht="15.75" customHeight="1"/>
+    <row r="1765" ht="15.75" customHeight="1"/>
+    <row r="1766" ht="15.75" customHeight="1"/>
+    <row r="1767" ht="15.75" customHeight="1"/>
+    <row r="1768" ht="15.75" customHeight="1"/>
+    <row r="1769" ht="15.75" customHeight="1"/>
+    <row r="1770" ht="15.75" customHeight="1"/>
+    <row r="1771" ht="15.75" customHeight="1"/>
+    <row r="1772" ht="15.75" customHeight="1"/>
+    <row r="1773" ht="15.75" customHeight="1"/>
+    <row r="1774" ht="15.75" customHeight="1"/>
+    <row r="1775" ht="15.75" customHeight="1"/>
+    <row r="1776" ht="15.75" customHeight="1"/>
+    <row r="1777" ht="15.75" customHeight="1"/>
+    <row r="1778" ht="15.75" customHeight="1"/>
+    <row r="1779" ht="15.75" customHeight="1"/>
+    <row r="1780" ht="15.75" customHeight="1"/>
+    <row r="1781" ht="15.75" customHeight="1"/>
+    <row r="1782" ht="15.75" customHeight="1"/>
+    <row r="1783" ht="15.75" customHeight="1"/>
+    <row r="1784" ht="15.75" customHeight="1"/>
+    <row r="1785" ht="15.75" customHeight="1"/>
+    <row r="1786" ht="15.75" customHeight="1"/>
+    <row r="1787" ht="15.75" customHeight="1"/>
+    <row r="1788" ht="15.75" customHeight="1"/>
+    <row r="1789" ht="15.75" customHeight="1"/>
+    <row r="1790" ht="15.75" customHeight="1"/>
+    <row r="1791" ht="15.75" customHeight="1"/>
+    <row r="1792" ht="15.75" customHeight="1"/>
+    <row r="1793" ht="15.75" customHeight="1"/>
+    <row r="1794" ht="15.75" customHeight="1"/>
+    <row r="1795" ht="15.75" customHeight="1"/>
+    <row r="1796" ht="15.75" customHeight="1"/>
+    <row r="1797" ht="15.75" customHeight="1"/>
+    <row r="1798" ht="15.75" customHeight="1"/>
+    <row r="1799" ht="15.75" customHeight="1"/>
+    <row r="1800" ht="15.75" customHeight="1"/>
+    <row r="1801" ht="15.75" customHeight="1"/>
+    <row r="1802" ht="15.75" customHeight="1"/>
+    <row r="1803" ht="15.75" customHeight="1"/>
+    <row r="1804" ht="15.75" customHeight="1"/>
+    <row r="1805" ht="15.75" customHeight="1"/>
+    <row r="1806" ht="15.75" customHeight="1"/>
+    <row r="1807" ht="15.75" customHeight="1"/>
+    <row r="1808" ht="15.75" customHeight="1"/>
+    <row r="1809" ht="15.75" customHeight="1"/>
+    <row r="1810" ht="15.75" customHeight="1"/>
+    <row r="1811" ht="15.75" customHeight="1"/>
+    <row r="1812" ht="15.75" customHeight="1"/>
+    <row r="1813" ht="15.75" customHeight="1"/>
+    <row r="1814" ht="15.75" customHeight="1"/>
+    <row r="1815" ht="15.75" customHeight="1"/>
+    <row r="1816" ht="15.75" customHeight="1"/>
+    <row r="1817" ht="15.75" customHeight="1"/>
+    <row r="1818" ht="15.75" customHeight="1"/>
+    <row r="1819" ht="15.75" customHeight="1"/>
+    <row r="1820" ht="15.75" customHeight="1"/>
+    <row r="1821" ht="15.75" customHeight="1"/>
+    <row r="1822" ht="15.75" customHeight="1"/>
+    <row r="1823" ht="15.75" customHeight="1"/>
+    <row r="1824" ht="15.75" customHeight="1"/>
+    <row r="1825" ht="15.75" customHeight="1"/>
+    <row r="1826" ht="15.75" customHeight="1"/>
+    <row r="1827" ht="15.75" customHeight="1"/>
+    <row r="1828" ht="15.75" customHeight="1"/>
+    <row r="1829" ht="15.75" customHeight="1"/>
+    <row r="1830" ht="15.75" customHeight="1"/>
+    <row r="1831" ht="15.75" customHeight="1"/>
+    <row r="1832" ht="15.75" customHeight="1"/>
+    <row r="1833" ht="15.75" customHeight="1"/>
+    <row r="1834" ht="15.75" customHeight="1"/>
+    <row r="1835" ht="15.75" customHeight="1"/>
+    <row r="1836" ht="15.75" customHeight="1"/>
+    <row r="1837" ht="15.75" customHeight="1"/>
+    <row r="1838" ht="15.75" customHeight="1"/>
+    <row r="1839" ht="15.75" customHeight="1"/>
+    <row r="1840" ht="15.75" customHeight="1"/>
+    <row r="1841" ht="15.75" customHeight="1"/>
+    <row r="1842" ht="15.75" customHeight="1"/>
+    <row r="1843" ht="15.75" customHeight="1"/>
+    <row r="1844" ht="15.75" customHeight="1"/>
+    <row r="1845" ht="15.75" customHeight="1"/>
+    <row r="1846" ht="15.75" customHeight="1"/>
+    <row r="1847" ht="15.75" customHeight="1"/>
+    <row r="1848" ht="15.75" customHeight="1"/>
+    <row r="1849" ht="15.75" customHeight="1"/>
+    <row r="1850" ht="15.75" customHeight="1"/>
+    <row r="1851" ht="15.75" customHeight="1"/>
+    <row r="1852" ht="15.75" customHeight="1"/>
+    <row r="1853" ht="15.75" customHeight="1"/>
+    <row r="1854" ht="15.75" customHeight="1"/>
+    <row r="1855" ht="15.75" customHeight="1"/>
+    <row r="1856" ht="15.75" customHeight="1"/>
+    <row r="1857" ht="15.75" customHeight="1"/>
+    <row r="1858" ht="15.75" customHeight="1"/>
+    <row r="1859" ht="15.75" customHeight="1"/>
+    <row r="1860" ht="15.75" customHeight="1"/>
+    <row r="1861" ht="15.75" customHeight="1"/>
+    <row r="1862" ht="15.75" customHeight="1"/>
+    <row r="1863" ht="15.75" customHeight="1"/>
+    <row r="1864" ht="15.75" customHeight="1"/>
+    <row r="1865" ht="15.75" customHeight="1"/>
+    <row r="1866" ht="15.75" customHeight="1"/>
+    <row r="1867" ht="15.75" customHeight="1"/>
+    <row r="1868" ht="15.75" customHeight="1"/>
+    <row r="1869" ht="15.75" customHeight="1"/>
+    <row r="1870" ht="15.75" customHeight="1"/>
+    <row r="1871" ht="15.75" customHeight="1"/>
+    <row r="1872" ht="15.75" customHeight="1"/>
+    <row r="1873" ht="15.75" customHeight="1"/>
+    <row r="1874" ht="15.75" customHeight="1"/>
+    <row r="1875" ht="15.75" customHeight="1"/>
+    <row r="1876" ht="15.75" customHeight="1"/>
+    <row r="1877" ht="15.75" customHeight="1"/>
+    <row r="1878" ht="15.75" customHeight="1"/>
+    <row r="1879" ht="15.75" customHeight="1"/>
+    <row r="1880" ht="15.75" customHeight="1"/>
+    <row r="1881" ht="15.75" customHeight="1"/>
+    <row r="1882" ht="15.75" customHeight="1"/>
+    <row r="1883" ht="15.75" customHeight="1"/>
+    <row r="1884" ht="15.75" customHeight="1"/>
+    <row r="1885" ht="15.75" customHeight="1"/>
+    <row r="1886" ht="15.75" customHeight="1"/>
+    <row r="1887" ht="15.75" customHeight="1"/>
+    <row r="1888" ht="15.75" customHeight="1"/>
+    <row r="1889" ht="15.75" customHeight="1"/>
+    <row r="1890" ht="15.75" customHeight="1"/>
+    <row r="1891" ht="15.75" customHeight="1"/>
+    <row r="1892" ht="15.75" customHeight="1"/>
+    <row r="1893" ht="15.75" customHeight="1"/>
+    <row r="1894" ht="15.75" customHeight="1"/>
+    <row r="1895" ht="15.75" customHeight="1"/>
+    <row r="1896" ht="15.75" customHeight="1"/>
+    <row r="1897" ht="15.75" customHeight="1"/>
+    <row r="1898" ht="15.75" customHeight="1"/>
+    <row r="1899" ht="15.75" customHeight="1"/>
+    <row r="1900" ht="15.75" customHeight="1"/>
+    <row r="1901" ht="15.75" customHeight="1"/>
+    <row r="1902" ht="15.75" customHeight="1"/>
+    <row r="1903" ht="15.75" customHeight="1"/>
+    <row r="1904" ht="15.75" customHeight="1"/>
+    <row r="1905" ht="15.75" customHeight="1"/>
+    <row r="1906" ht="15.75" customHeight="1"/>
+    <row r="1907" ht="15.75" customHeight="1"/>
+    <row r="1908" ht="15.75" customHeight="1"/>
+    <row r="1909" ht="15.75" customHeight="1"/>
+    <row r="1910" ht="15.75" customHeight="1"/>
+    <row r="1911" ht="15.75" customHeight="1"/>
+    <row r="1912" ht="15.75" customHeight="1"/>
+    <row r="1913" ht="15.75" customHeight="1"/>
+    <row r="1914" ht="15.75" customHeight="1"/>
+    <row r="1915" ht="15.75" customHeight="1"/>
+    <row r="1916" ht="15.75" customHeight="1"/>
+    <row r="1917" ht="15.75" customHeight="1"/>
+    <row r="1918" ht="15.75" customHeight="1"/>
+    <row r="1919" ht="15.75" customHeight="1"/>
+    <row r="1920" ht="15.75" customHeight="1"/>
+    <row r="1921" ht="15.75" customHeight="1"/>
+    <row r="1922" ht="15.75" customHeight="1"/>
+    <row r="1923" ht="15.75" customHeight="1"/>
+    <row r="1924" ht="15.75" customHeight="1"/>
+    <row r="1925" ht="15.75" customHeight="1"/>
+    <row r="1926" ht="15.75" customHeight="1"/>
+    <row r="1927" ht="15.75" customHeight="1"/>
+    <row r="1928" ht="15.75" customHeight="1"/>
+    <row r="1929" ht="15.75" customHeight="1"/>
+    <row r="1930" ht="15.75" customHeight="1"/>
+    <row r="1931" ht="15.75" customHeight="1"/>
+    <row r="1932" ht="15.75" customHeight="1"/>
+    <row r="1933" ht="15.75" customHeight="1"/>
+    <row r="1934" ht="15.75" customHeight="1"/>
+    <row r="1935" ht="15.75" customHeight="1"/>
+    <row r="1936" ht="15.75" customHeight="1"/>
+    <row r="1937" ht="15.75" customHeight="1"/>
+    <row r="1938" ht="15.75" customHeight="1"/>
+    <row r="1939" ht="15.75" customHeight="1"/>
+    <row r="1940" ht="15.75" customHeight="1"/>
+    <row r="1941" ht="15.75" customHeight="1"/>
+    <row r="1942" ht="15.75" customHeight="1"/>
+    <row r="1943" ht="15.75" customHeight="1"/>
+    <row r="1944" ht="15.75" customHeight="1"/>
+    <row r="1945" ht="15.75" customHeight="1"/>
+    <row r="1946" ht="15.75" customHeight="1"/>
+    <row r="1947" ht="15.75" customHeight="1"/>
+    <row r="1948" ht="15.75" customHeight="1"/>
+    <row r="1949" ht="15.75" customHeight="1"/>
+    <row r="1950" ht="15.75" customHeight="1"/>
+    <row r="1951" ht="15.75" customHeight="1"/>
+    <row r="1952" ht="15.75" customHeight="1"/>
+    <row r="1953" ht="15.75" customHeight="1"/>
+    <row r="1954" ht="15.75" customHeight="1"/>
+    <row r="1955" ht="15.75" customHeight="1"/>
+    <row r="1956" ht="15.75" customHeight="1"/>
+    <row r="1957" ht="15.75" customHeight="1"/>
+    <row r="1958" ht="15.75" customHeight="1"/>
+    <row r="1959" ht="15.75" customHeight="1"/>
+    <row r="1960" ht="15.75" customHeight="1"/>
+    <row r="1961" ht="15.75" customHeight="1"/>
+    <row r="1962" ht="15.75" customHeight="1"/>
+    <row r="1963" ht="15.75" customHeight="1"/>
+    <row r="1964" ht="15.75" customHeight="1"/>
+    <row r="1965" ht="15.75" customHeight="1"/>
+    <row r="1966" ht="15.75" customHeight="1"/>
+    <row r="1967" ht="15.75" customHeight="1"/>
+    <row r="1968" ht="15.75" customHeight="1"/>
+    <row r="1969" ht="15.75" customHeight="1"/>
+    <row r="1970" ht="15.75" customHeight="1"/>
+    <row r="1971" ht="15.75" customHeight="1"/>
+    <row r="1972" ht="15.75" customHeight="1"/>
+    <row r="1973" ht="15.75" customHeight="1"/>
+    <row r="1974" ht="15.75" customHeight="1"/>
+    <row r="1975" ht="15.75" customHeight="1"/>
+    <row r="1976" ht="15.75" customHeight="1"/>
+    <row r="1977" ht="15.75" customHeight="1"/>
+    <row r="1978" ht="15.75" customHeight="1"/>
+    <row r="1979" ht="15.75" customHeight="1"/>
+    <row r="1980" ht="15.75" customHeight="1"/>
+    <row r="1981" ht="15.75" customHeight="1"/>
+    <row r="1982" ht="15.75" customHeight="1"/>
+    <row r="1983" ht="15.75" customHeight="1"/>
+    <row r="1984" ht="15.75" customHeight="1"/>
+    <row r="1985" ht="15.75" customHeight="1"/>
+    <row r="1986" ht="15.75" customHeight="1"/>
+    <row r="1987" ht="15.75" customHeight="1"/>
+    <row r="1988" ht="15.75" customHeight="1"/>
+    <row r="1989" ht="15.75" customHeight="1"/>
+    <row r="1990" ht="15.75" customHeight="1"/>
+    <row r="1991" ht="15.75" customHeight="1"/>
+    <row r="1992" ht="15.75" customHeight="1"/>
+    <row r="1993" ht="15.75" customHeight="1"/>
+    <row r="1994" ht="15.75" customHeight="1"/>
+    <row r="1995" ht="15.75" customHeight="1"/>
+    <row r="1996" ht="15.75" customHeight="1"/>
+    <row r="1997" ht="15.75" customHeight="1"/>
+    <row r="1998" ht="15.75" customHeight="1"/>
+    <row r="1999" ht="15.75" customHeight="1"/>
+    <row r="2000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$2:$J$27"/>
   <mergeCells count="5">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A10:J10"/>
     <mergeCell ref="A15:J15"/>
     <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A10:J10"/>
-    <mergeCell ref="A3:J3"/>
   </mergeCells>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H9 H11:H14 H16:H19 H21">
+      <formula1>"Fail,Pass"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
@@ -5192,7 +6240,7 @@
       <c r="G2" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="18" t="s">
         <v>41</v>
       </c>
       <c r="I2" s="5" t="s">
@@ -5203,7 +6251,7 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="37" t="s">
         <v>155</v>
       </c>
       <c r="B3" s="15"/>
@@ -5217,692 +6265,729 @@
       <c r="J3" s="16"/>
     </row>
     <row r="4" ht="69.75" customHeight="1">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="38" t="s">
         <v>158</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="38" t="s">
         <v>160</v>
       </c>
-      <c r="G4" s="37"/>
-      <c r="H4" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" s="38" t="s">
+      <c r="G4" s="38"/>
+      <c r="H4" s="39" t="s">
+        <v>161</v>
+      </c>
+      <c r="I4" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="37" t="s">
-        <v>161</v>
+      <c r="J4" s="38" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1">
       <c r="A5" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G5" s="13"/>
-      <c r="H5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I5" s="38" t="s">
+      <c r="H5" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" ht="69.75" customHeight="1">
-      <c r="A6" s="37" t="s">
-        <v>169</v>
-      </c>
-      <c r="B6" s="37" t="s">
+      <c r="A6" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="C6" s="37" t="s">
+      <c r="B6" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="C6" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="E6" s="37" t="s">
+      <c r="D6" s="38" t="s">
         <v>173</v>
       </c>
-      <c r="F6" s="37" t="s">
+      <c r="E6" s="38" t="s">
         <v>174</v>
       </c>
-      <c r="G6" s="37"/>
-      <c r="H6" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="38" t="s">
+      <c r="F6" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="38"/>
+      <c r="H6" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I6" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="37" t="s">
-        <v>175</v>
+      <c r="J6" s="38" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="7" ht="69.75" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G7" s="13"/>
-      <c r="H7" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I7" s="38" t="s">
+      <c r="H7" s="39" t="s">
+        <v>161</v>
+      </c>
+      <c r="I7" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" ht="69.75" customHeight="1">
-      <c r="A8" s="37" t="s">
-        <v>182</v>
-      </c>
-      <c r="B8" s="37" t="s">
+      <c r="A8" s="38" t="s">
         <v>183</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="B8" s="38" t="s">
         <v>184</v>
       </c>
-      <c r="D8" s="37" t="s">
+      <c r="C8" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="E8" s="37" t="s">
+      <c r="D8" s="38" t="s">
         <v>186</v>
       </c>
-      <c r="F8" s="37" t="s">
+      <c r="E8" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I8" s="38" t="s">
+      <c r="F8" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="G8" s="38"/>
+      <c r="H8" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I8" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J8" s="37" t="s">
-        <v>188</v>
+      <c r="J8" s="38" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="9" ht="69.75" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I9" s="38" t="s">
+        <v>195</v>
+      </c>
+      <c r="G9" s="42"/>
+      <c r="H9" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I9" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10" ht="69.75" customHeight="1">
-      <c r="A10" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="B10" s="37" t="s">
+      <c r="A10" s="38" t="s">
         <v>197</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="B10" s="38" t="s">
         <v>198</v>
       </c>
-      <c r="D10" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="E10" s="37" t="s">
+      <c r="C10" s="38" t="s">
         <v>199</v>
       </c>
-      <c r="F10" s="37" t="s">
+      <c r="D10" s="38" t="s">
+        <v>166</v>
+      </c>
+      <c r="E10" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="G10" s="37"/>
-      <c r="H10" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I10" s="38" t="s">
+      <c r="F10" s="38" t="s">
+        <v>201</v>
+      </c>
+      <c r="G10" s="38"/>
+      <c r="H10" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I10" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J10" s="37" t="s">
-        <v>201</v>
+      <c r="J10" s="38" t="s">
+        <v>202</v>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="36" t="s">
-        <v>202</v>
-      </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="16"/>
+    <row r="11" ht="69.75" customHeight="1">
+      <c r="A11" s="38" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>206</v>
+      </c>
+      <c r="F11" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38" t="s">
+        <v>207</v>
+      </c>
+      <c r="I11" s="38" t="s">
+        <v>208</v>
+      </c>
+      <c r="J11" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+      <c r="Q11" s="43"/>
+      <c r="R11" s="43"/>
     </row>
-    <row r="12" ht="69.75" customHeight="1">
+    <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="37" t="s">
-        <v>203</v>
-      </c>
-      <c r="B12" s="37" t="s">
-        <v>204</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>205</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>206</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>207</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>208</v>
-      </c>
-      <c r="G12" s="37"/>
-      <c r="H12" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I12" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="J12" s="37" t="s">
-        <v>209</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="16"/>
     </row>
     <row r="13" ht="69.75" customHeight="1">
-      <c r="A13" s="13" t="s">
-        <v>210</v>
-      </c>
-      <c r="B13" s="13" t="s">
+      <c r="A13" s="38" t="s">
+        <v>203</v>
+      </c>
+      <c r="B13" s="38" t="s">
         <v>211</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="38" t="s">
         <v>212</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="38" t="s">
         <v>214</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="38" t="s">
         <v>215</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I13" s="38" t="s">
+      <c r="G13" s="38"/>
+      <c r="H13" s="39" t="s">
+        <v>161</v>
+      </c>
+      <c r="I13" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J13" s="13" t="s">
+      <c r="J13" s="38" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="14" ht="69.75" customHeight="1">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="C14" s="37" t="s">
+      <c r="C14" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="D14" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="E14" s="37" t="s">
+      <c r="E14" s="13" t="s">
         <v>221</v>
       </c>
-      <c r="F14" s="37" t="s">
+      <c r="F14" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="G14" s="37"/>
-      <c r="H14" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I14" s="38" t="s">
+      <c r="G14" s="13"/>
+      <c r="H14" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I14" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J14" s="37" t="s">
+      <c r="J14" s="13" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="15" ht="69.75" customHeight="1">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="38" t="s">
         <v>224</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="38" t="s">
         <v>225</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="38" t="s">
         <v>226</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="38" t="s">
         <v>227</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="38" t="s">
         <v>228</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I15" s="38" t="s">
+      <c r="G15" s="38"/>
+      <c r="H15" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I15" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J15" s="13" t="s">
+      <c r="J15" s="38" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="16" ht="69.75" customHeight="1">
-      <c r="A16" s="37" t="s">
+      <c r="A16" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="C16" s="37" t="s">
+      <c r="C16" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="E16" s="37" t="s">
+      <c r="E16" s="13" t="s">
         <v>235</v>
       </c>
-      <c r="F16" s="37" t="s">
+      <c r="F16" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="G16" s="37"/>
-      <c r="H16" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I16" s="39" t="s">
+      <c r="G16" s="13"/>
+      <c r="H16" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I16" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="J16" s="13" t="s">
         <v>237</v>
-      </c>
-      <c r="J16" s="37" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="17" ht="69.75" customHeight="1">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="38" t="s">
+        <v>238</v>
+      </c>
+      <c r="B17" s="38" t="s">
         <v>239</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="C17" s="38" t="s">
         <v>240</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="D17" s="38" t="s">
         <v>241</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="E17" s="38" t="s">
         <v>242</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="F17" s="38" t="s">
         <v>243</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="G17" s="38"/>
+      <c r="H17" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="I17" s="45" t="s">
         <v>244</v>
       </c>
-      <c r="G17" s="13"/>
-      <c r="H17" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I17" s="39" t="s">
-        <v>237</v>
-      </c>
-      <c r="J17" s="13" t="s">
+      <c r="J17" s="38" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="18" ht="69.75" customHeight="1">
-      <c r="A18" s="37" t="s">
+      <c r="A18" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="B18" s="37" t="s">
+      <c r="B18" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="C18" s="37" t="s">
+      <c r="C18" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="D18" s="37" t="s">
+      <c r="D18" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="E18" s="37" t="s">
+      <c r="E18" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="F18" s="37" t="s">
+      <c r="F18" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="G18" s="37"/>
-      <c r="H18" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I18" s="38" t="s">
+      <c r="G18" s="13"/>
+      <c r="H18" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="I18" s="45" t="s">
+        <v>244</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="19" ht="69.75" customHeight="1">
+      <c r="A19" s="38" t="s">
+        <v>253</v>
+      </c>
+      <c r="B19" s="38" t="s">
+        <v>254</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>255</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>256</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>257</v>
+      </c>
+      <c r="F19" s="38" t="s">
+        <v>258</v>
+      </c>
+      <c r="G19" s="38"/>
+      <c r="H19" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I19" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J18" s="37" t="s">
-        <v>252</v>
+      <c r="J19" s="38" t="s">
+        <v>259</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="36" t="s">
-        <v>253</v>
-      </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="16"/>
-    </row>
-    <row r="20" ht="69.75" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="B20" s="37" t="s">
-        <v>255</v>
-      </c>
-      <c r="C20" s="37" t="s">
-        <v>256</v>
-      </c>
-      <c r="D20" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="E20" s="37" t="s">
-        <v>257</v>
-      </c>
-      <c r="F20" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="G20" s="37"/>
-      <c r="H20" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I20" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="J20" s="37" t="s">
-        <v>259</v>
-      </c>
+        <v>260</v>
+      </c>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="16"/>
     </row>
     <row r="21" ht="69.75" customHeight="1">
-      <c r="A21" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="B21" s="13" t="s">
+      <c r="A21" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="B21" s="38" t="s">
         <v>262</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="C21" s="38" t="s">
         <v>263</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="D21" s="38" t="s">
+        <v>166</v>
+      </c>
+      <c r="E21" s="38" t="s">
         <v>264</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="F21" s="38" t="s">
         <v>265</v>
       </c>
-      <c r="G21" s="13"/>
-      <c r="H21" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I21" s="38" t="s">
+      <c r="G21" s="38"/>
+      <c r="H21" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I21" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J21" s="13" t="s">
+      <c r="J21" s="38" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="36" t="s">
+    <row r="22" ht="69.75" customHeight="1">
+      <c r="A22" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="16"/>
+      <c r="B22" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>272</v>
+      </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I22" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>273</v>
+      </c>
     </row>
-    <row r="23" ht="69.75" customHeight="1">
-      <c r="A23" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>269</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>270</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="G23" s="13"/>
-      <c r="H23" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I23" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="J23" s="13" t="s">
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="37" t="s">
         <v>274</v>
       </c>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="16"/>
     </row>
     <row r="24" ht="69.75" customHeight="1">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="13" t="s">
         <v>275</v>
       </c>
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="13" t="s">
         <v>276</v>
       </c>
-      <c r="C24" s="37" t="s">
+      <c r="C24" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="D24" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="E24" s="37" t="s">
+      <c r="D24" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="F24" s="37" t="s">
+      <c r="E24" s="13" t="s">
         <v>279</v>
       </c>
-      <c r="G24" s="37"/>
-      <c r="H24" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I24" s="38" t="s">
+      <c r="F24" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="G24" s="13"/>
+      <c r="H24" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I24" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J24" s="37" t="s">
-        <v>280</v>
+      <c r="J24" s="13" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="25" ht="69.75" customHeight="1">
-      <c r="A25" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="B25" s="13" t="s">
+      <c r="A25" s="38" t="s">
         <v>282</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="B25" s="38" t="s">
         <v>283</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="C25" s="38" t="s">
+        <v>284</v>
+      </c>
+      <c r="D25" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="13" t="s">
-        <v>284</v>
-      </c>
-      <c r="F25" s="13" t="s">
+      <c r="E25" s="38" t="s">
         <v>285</v>
       </c>
-      <c r="G25" s="13"/>
-      <c r="H25" s="10" t="s">
-        <v>7</v>
+      <c r="F25" s="38" t="s">
+        <v>286</v>
+      </c>
+      <c r="G25" s="38"/>
+      <c r="H25" s="41" t="s">
+        <v>161</v>
       </c>
       <c r="I25" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="J25" s="38" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="26" ht="69.75" customHeight="1">
+      <c r="A26" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="G26" s="13"/>
+      <c r="H26" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="I26" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="J25" s="13" t="s">
-        <v>286</v>
+      <c r="J26" s="13" t="s">
+        <v>293</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="36" t="s">
-        <v>287</v>
-      </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="16"/>
-    </row>
-    <row r="27" ht="69.75" customHeight="1">
-      <c r="A27" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>290</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>291</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>292</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="G27" s="13"/>
-      <c r="H27" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I27" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="J27" s="13" t="s">
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="37" t="s">
         <v>294</v>
       </c>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="16"/>
     </row>
     <row r="28" ht="69.75" customHeight="1">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="13" t="s">
         <v>295</v>
       </c>
-      <c r="B28" s="37" t="s">
+      <c r="B28" s="13" t="s">
         <v>296</v>
       </c>
-      <c r="C28" s="37" t="s">
+      <c r="C28" s="13" t="s">
         <v>297</v>
       </c>
-      <c r="D28" s="37" t="s">
+      <c r="D28" s="13" t="s">
         <v>298</v>
       </c>
-      <c r="E28" s="37" t="s">
+      <c r="E28" s="13" t="s">
         <v>299</v>
       </c>
-      <c r="F28" s="37" t="s">
+      <c r="F28" s="13" t="s">
         <v>300</v>
       </c>
-      <c r="G28" s="37"/>
-      <c r="H28" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="I28" s="38" t="s">
+      <c r="G28" s="13"/>
+      <c r="H28" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I28" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J28" s="37" t="s">
+      <c r="J28" s="13" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="29" ht="69.75" customHeight="1">
+      <c r="A29" s="38" t="s">
+        <v>302</v>
+      </c>
+      <c r="B29" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="E29" s="38" t="s">
+        <v>306</v>
+      </c>
+      <c r="F29" s="38" t="s">
+        <v>307</v>
+      </c>
+      <c r="G29" s="38"/>
+      <c r="H29" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="I29" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="J29" s="38" t="s">
+        <v>308</v>
+      </c>
+    </row>
     <row r="30" ht="15.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
@@ -6874,21 +7959,22 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$2:$J$28"/>
+  <autoFilter ref="$A$2:$J$29"/>
   <mergeCells count="6">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A19:J19"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A27:J27"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H10 H12:H18 H20:H21 H23:H25 H27:H28">
-      <formula1>"Đạt,Không đạt"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H4:H11 H13:H19 H21:H22 H24:H26 H28:H29">
+      <formula1>"Failed,Passed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I4:I10 I12:I18 I20:I21 I23:I25 I27:I28">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I4:I11 I13:I19 I21:I22 I24:I26 I28:I29">
       <formula1>"Không có,Thấp,Cao"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6921,7 +8007,7 @@
   <sheetData>
     <row r="1" ht="25.5" customHeight="1">
       <c r="A1" s="17" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6966,7 +8052,7 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="37" t="s">
         <v>155</v>
       </c>
       <c r="B3" s="15"/>
@@ -6980,218 +8066,218 @@
       <c r="J3" s="16"/>
     </row>
     <row r="4" ht="69.75" customHeight="1">
-      <c r="A4" s="37" t="s">
-        <v>303</v>
-      </c>
-      <c r="B4" s="37" t="s">
-        <v>304</v>
-      </c>
-      <c r="C4" s="37" t="s">
-        <v>305</v>
-      </c>
-      <c r="D4" s="37" t="s">
+      <c r="A4" s="38" t="s">
+        <v>310</v>
+      </c>
+      <c r="B4" s="38" t="s">
+        <v>311</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>312</v>
+      </c>
+      <c r="D4" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="37" t="s">
-        <v>306</v>
-      </c>
-      <c r="F4" s="37" t="s">
-        <v>307</v>
-      </c>
-      <c r="G4" s="37"/>
+      <c r="E4" s="38" t="s">
+        <v>313</v>
+      </c>
+      <c r="F4" s="38" t="s">
+        <v>314</v>
+      </c>
+      <c r="G4" s="38"/>
       <c r="H4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="38" t="s">
+      <c r="I4" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="37" t="s">
-        <v>308</v>
+      <c r="J4" s="38" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="5" ht="69.75" customHeight="1">
       <c r="A5" s="13" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="G5" s="13"/>
       <c r="H5" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="38" t="s">
+      <c r="I5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" ht="69.75" customHeight="1">
-      <c r="A6" s="37" t="s">
-        <v>316</v>
-      </c>
-      <c r="B6" s="37" t="s">
-        <v>317</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>318</v>
-      </c>
-      <c r="D6" s="37" t="s">
-        <v>319</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>320</v>
-      </c>
-      <c r="F6" s="37" t="s">
-        <v>174</v>
-      </c>
-      <c r="G6" s="37"/>
+      <c r="A6" s="38" t="s">
+        <v>323</v>
+      </c>
+      <c r="B6" s="38" t="s">
+        <v>324</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>325</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>326</v>
+      </c>
+      <c r="E6" s="38" t="s">
+        <v>327</v>
+      </c>
+      <c r="F6" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="38"/>
       <c r="H6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="38" t="s">
+      <c r="I6" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="37" t="s">
-        <v>321</v>
+      <c r="J6" s="38" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="7" ht="69.75" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="G7" s="13"/>
       <c r="H7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="38" t="s">
+      <c r="I7" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="8" ht="69.75" customHeight="1">
-      <c r="A8" s="37" t="s">
-        <v>329</v>
-      </c>
-      <c r="B8" s="37" t="s">
-        <v>330</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>331</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>332</v>
-      </c>
-      <c r="E8" s="37" t="s">
-        <v>333</v>
-      </c>
-      <c r="F8" s="37" t="s">
-        <v>334</v>
-      </c>
-      <c r="G8" s="37"/>
+      <c r="A8" s="38" t="s">
+        <v>336</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>337</v>
+      </c>
+      <c r="C8" s="38" t="s">
+        <v>338</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>339</v>
+      </c>
+      <c r="E8" s="38" t="s">
+        <v>340</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>341</v>
+      </c>
+      <c r="G8" s="38"/>
       <c r="H8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I8" s="38" t="s">
+      <c r="I8" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J8" s="37" t="s">
-        <v>335</v>
+      <c r="J8" s="38" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="9" ht="69.75" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>48</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="G9" s="13"/>
       <c r="H9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I9" s="38" t="s">
+      <c r="I9" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10" ht="69.75" customHeight="1">
-      <c r="A10" s="37" t="s">
-        <v>342</v>
-      </c>
-      <c r="B10" s="37" t="s">
-        <v>343</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>344</v>
-      </c>
-      <c r="D10" s="37" t="s">
+      <c r="A10" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="B10" s="38" t="s">
+        <v>350</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>351</v>
+      </c>
+      <c r="D10" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="37" t="s">
-        <v>345</v>
-      </c>
-      <c r="F10" s="37" t="s">
-        <v>346</v>
-      </c>
-      <c r="G10" s="37"/>
+      <c r="E10" s="38" t="s">
+        <v>352</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>353</v>
+      </c>
+      <c r="G10" s="38"/>
       <c r="H10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I10" s="38" t="s">
+      <c r="I10" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J10" s="37" t="s">
-        <v>347</v>
+      <c r="J10" s="38" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="36" t="s">
-        <v>348</v>
+      <c r="A11" s="37" t="s">
+        <v>355</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
@@ -7204,218 +8290,218 @@
       <c r="J11" s="16"/>
     </row>
     <row r="12" ht="69.75" customHeight="1">
-      <c r="A12" s="37" t="s">
-        <v>349</v>
-      </c>
-      <c r="B12" s="37" t="s">
-        <v>350</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>351</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>352</v>
-      </c>
-      <c r="E12" s="37" t="s">
-        <v>353</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>354</v>
-      </c>
-      <c r="G12" s="37"/>
+      <c r="A12" s="38" t="s">
+        <v>356</v>
+      </c>
+      <c r="B12" s="38" t="s">
+        <v>357</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>358</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>359</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>360</v>
+      </c>
+      <c r="F12" s="38" t="s">
+        <v>361</v>
+      </c>
+      <c r="G12" s="38"/>
       <c r="H12" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="38" t="s">
+      <c r="I12" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J12" s="37" t="s">
-        <v>355</v>
+      <c r="J12" s="38" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="13" ht="69.75" customHeight="1">
       <c r="A13" s="13" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="G13" s="13"/>
       <c r="H13" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I13" s="40" t="s">
+      <c r="I13" s="46" t="s">
         <v>103</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
     </row>
     <row r="14" ht="69.75" customHeight="1">
-      <c r="A14" s="37" t="s">
-        <v>363</v>
-      </c>
-      <c r="B14" s="37" t="s">
-        <v>364</v>
-      </c>
-      <c r="C14" s="37" t="s">
-        <v>365</v>
-      </c>
-      <c r="D14" s="37" t="s">
-        <v>366</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>367</v>
-      </c>
-      <c r="F14" s="37" t="s">
-        <v>368</v>
-      </c>
-      <c r="G14" s="37"/>
+      <c r="A14" s="38" t="s">
+        <v>370</v>
+      </c>
+      <c r="B14" s="38" t="s">
+        <v>371</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>372</v>
+      </c>
+      <c r="D14" s="38" t="s">
+        <v>373</v>
+      </c>
+      <c r="E14" s="38" t="s">
+        <v>374</v>
+      </c>
+      <c r="F14" s="38" t="s">
+        <v>375</v>
+      </c>
+      <c r="G14" s="38"/>
       <c r="H14" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I14" s="38" t="s">
+      <c r="I14" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J14" s="37" t="s">
-        <v>369</v>
+      <c r="J14" s="38" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="15" ht="69.75" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="G15" s="13"/>
       <c r="H15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I15" s="38" t="s">
+      <c r="I15" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
     </row>
     <row r="16" ht="69.75" customHeight="1">
-      <c r="A16" s="37" t="s">
-        <v>377</v>
-      </c>
-      <c r="B16" s="37" t="s">
-        <v>378</v>
-      </c>
-      <c r="C16" s="37" t="s">
-        <v>379</v>
-      </c>
-      <c r="D16" s="37" t="s">
-        <v>380</v>
-      </c>
-      <c r="E16" s="37" t="s">
-        <v>381</v>
-      </c>
-      <c r="F16" s="37" t="s">
-        <v>382</v>
-      </c>
-      <c r="G16" s="37"/>
+      <c r="A16" s="38" t="s">
+        <v>384</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>385</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>386</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>387</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>388</v>
+      </c>
+      <c r="F16" s="38" t="s">
+        <v>389</v>
+      </c>
+      <c r="G16" s="38"/>
       <c r="H16" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I16" s="40" t="s">
+      <c r="I16" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="J16" s="37" t="s">
-        <v>383</v>
+      <c r="J16" s="38" t="s">
+        <v>390</v>
       </c>
     </row>
     <row r="17" ht="69.75" customHeight="1">
       <c r="A17" s="13" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I17" s="38" t="s">
+      <c r="I17" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
     </row>
     <row r="18" ht="69.75" customHeight="1">
-      <c r="A18" s="37" t="s">
-        <v>391</v>
-      </c>
-      <c r="B18" s="37" t="s">
-        <v>392</v>
-      </c>
-      <c r="C18" s="37" t="s">
-        <v>393</v>
-      </c>
-      <c r="D18" s="37" t="s">
-        <v>394</v>
-      </c>
-      <c r="E18" s="37" t="s">
-        <v>395</v>
-      </c>
-      <c r="F18" s="37" t="s">
-        <v>396</v>
-      </c>
-      <c r="G18" s="37"/>
+      <c r="A18" s="38" t="s">
+        <v>398</v>
+      </c>
+      <c r="B18" s="38" t="s">
+        <v>399</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>400</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>401</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>402</v>
+      </c>
+      <c r="F18" s="38" t="s">
+        <v>403</v>
+      </c>
+      <c r="G18" s="38"/>
       <c r="H18" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I18" s="38" t="s">
+      <c r="I18" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J18" s="37" t="s">
-        <v>397</v>
+      <c r="J18" s="38" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="36" t="s">
-        <v>398</v>
+      <c r="A19" s="37" t="s">
+        <v>405</v>
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -7428,68 +8514,68 @@
       <c r="J19" s="16"/>
     </row>
     <row r="20" ht="69.75" customHeight="1">
-      <c r="A20" s="37" t="s">
-        <v>399</v>
-      </c>
-      <c r="B20" s="37" t="s">
-        <v>400</v>
-      </c>
-      <c r="C20" s="37" t="s">
-        <v>401</v>
-      </c>
-      <c r="D20" s="37" t="s">
-        <v>402</v>
-      </c>
-      <c r="E20" s="37" t="s">
-        <v>403</v>
-      </c>
-      <c r="F20" s="37" t="s">
-        <v>404</v>
-      </c>
-      <c r="G20" s="37"/>
+      <c r="A20" s="38" t="s">
+        <v>406</v>
+      </c>
+      <c r="B20" s="38" t="s">
+        <v>407</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>408</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>409</v>
+      </c>
+      <c r="E20" s="38" t="s">
+        <v>410</v>
+      </c>
+      <c r="F20" s="38" t="s">
+        <v>411</v>
+      </c>
+      <c r="G20" s="38"/>
       <c r="H20" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I20" s="38" t="s">
+      <c r="I20" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J20" s="37" t="s">
-        <v>405</v>
+      <c r="J20" s="38" t="s">
+        <v>412</v>
       </c>
     </row>
     <row r="21" ht="69.75" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="G21" s="13"/>
       <c r="H21" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I21" s="38" t="s">
+      <c r="I21" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="36" t="s">
-        <v>413</v>
+      <c r="A22" s="37" t="s">
+        <v>420</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -7503,67 +8589,67 @@
     </row>
     <row r="23" ht="69.75" customHeight="1">
       <c r="A23" s="13" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="G23" s="13"/>
       <c r="H23" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I23" s="38" t="s">
+      <c r="I23" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
     </row>
     <row r="24" ht="69.75" customHeight="1">
-      <c r="A24" s="37" t="s">
-        <v>421</v>
-      </c>
-      <c r="B24" s="37" t="s">
-        <v>422</v>
-      </c>
-      <c r="C24" s="37" t="s">
-        <v>423</v>
-      </c>
-      <c r="D24" s="37" t="s">
+      <c r="A24" s="38" t="s">
+        <v>428</v>
+      </c>
+      <c r="B24" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C24" s="38" t="s">
+        <v>430</v>
+      </c>
+      <c r="D24" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="37" t="s">
-        <v>424</v>
-      </c>
-      <c r="F24" s="37" t="s">
-        <v>425</v>
-      </c>
-      <c r="G24" s="37"/>
+      <c r="E24" s="38" t="s">
+        <v>431</v>
+      </c>
+      <c r="F24" s="38" t="s">
+        <v>432</v>
+      </c>
+      <c r="G24" s="38"/>
       <c r="H24" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I24" s="38" t="s">
+      <c r="I24" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J24" s="37" t="s">
-        <v>426</v>
+      <c r="J24" s="38" t="s">
+        <v>433</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="36" t="s">
-        <v>427</v>
+      <c r="A25" s="37" t="s">
+        <v>434</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -7576,123 +8662,123 @@
       <c r="J25" s="16"/>
     </row>
     <row r="26" ht="69.75" customHeight="1">
-      <c r="A26" s="37" t="s">
-        <v>428</v>
-      </c>
-      <c r="B26" s="37" t="s">
-        <v>429</v>
-      </c>
-      <c r="C26" s="37" t="s">
-        <v>430</v>
-      </c>
-      <c r="D26" s="37" t="s">
-        <v>431</v>
-      </c>
-      <c r="E26" s="37" t="s">
-        <v>432</v>
-      </c>
-      <c r="F26" s="37" t="s">
-        <v>433</v>
-      </c>
-      <c r="G26" s="37"/>
+      <c r="A26" s="38" t="s">
+        <v>435</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>436</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>437</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>438</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>439</v>
+      </c>
+      <c r="F26" s="38" t="s">
+        <v>440</v>
+      </c>
+      <c r="G26" s="38"/>
       <c r="H26" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I26" s="38" t="s">
+      <c r="I26" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J26" s="37" t="s">
-        <v>294</v>
+      <c r="J26" s="38" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="27" ht="69.75" customHeight="1">
       <c r="A27" s="13" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="G27" s="13"/>
       <c r="H27" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I27" s="38" t="s">
+      <c r="I27" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
     </row>
     <row r="28" ht="69.75" customHeight="1">
-      <c r="A28" s="37" t="s">
-        <v>441</v>
-      </c>
-      <c r="B28" s="37" t="s">
-        <v>442</v>
-      </c>
-      <c r="C28" s="37" t="s">
-        <v>443</v>
-      </c>
-      <c r="D28" s="37" t="s">
-        <v>444</v>
-      </c>
-      <c r="E28" s="37" t="s">
-        <v>445</v>
-      </c>
-      <c r="F28" s="37" t="s">
-        <v>446</v>
-      </c>
-      <c r="G28" s="37"/>
+      <c r="A28" s="38" t="s">
+        <v>448</v>
+      </c>
+      <c r="B28" s="38" t="s">
+        <v>449</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>450</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>451</v>
+      </c>
+      <c r="E28" s="38" t="s">
+        <v>452</v>
+      </c>
+      <c r="F28" s="38" t="s">
+        <v>453</v>
+      </c>
+      <c r="G28" s="38"/>
       <c r="H28" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I28" s="38" t="s">
+      <c r="I28" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="J28" s="37" t="s">
-        <v>447</v>
+      <c r="J28" s="38" t="s">
+        <v>454</v>
       </c>
     </row>
     <row r="29" ht="69.75" customHeight="1">
       <c r="A29" s="13" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>48</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="G29" s="13"/>
       <c r="H29" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I29" s="38" t="s">
+      <c r="I29" s="40" t="s">
         <v>52</v>
       </c>
       <c r="J29" s="13" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Enhance test case ID normalization logic in testcase-loader
</commit_message>
<xml_diff>
--- a/Testcase-OrangeHRM.xlsx
+++ b/Testcase-OrangeHRM.xlsx
@@ -769,7 +769,7 @@
     <t>Dòng 3=tên tài khoản, dòng 4=vai trò, dòng 5=trạng thái, dòng 6=tên nhân viên</t>
   </si>
   <si>
-    <t>TC-U010</t>
+    <t>TC-U10</t>
   </si>
   <si>
     <t>Thêm người dùng với vai trò Quản trị viên</t>
@@ -1717,10 +1717,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="32">
     <font>
@@ -1819,9 +1819,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1829,6 +1859,59 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1851,45 +1934,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1897,15 +1942,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1915,43 +1952,6 @@
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2030,7 +2030,169 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2042,175 +2204,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2359,21 +2359,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -2394,21 +2379,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2442,8 +2412,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2451,150 +2421,180 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="15" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="38" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">

</xml_diff>